<commit_message>
Daily pulse data: 2026-09-06
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE139"/>
+  <dimension ref="A1:AE140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22295,6 +22295,163 @@
         </is>
       </c>
     </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>29116215991.989517</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>1987578808.439965</t>
+        </is>
+      </c>
+      <c r="D140" s="2" t="inlineStr">
+        <is>
+          <t>80342</t>
+        </is>
+      </c>
+      <c r="E140" s="2" t="inlineStr">
+        <is>
+          <t>1987215170.053582</t>
+        </is>
+      </c>
+      <c r="F140" s="2" t="inlineStr">
+        <is>
+          <t>22830215855.219997</t>
+        </is>
+      </c>
+      <c r="G140" s="2" t="inlineStr">
+        <is>
+          <t>375640</t>
+        </is>
+      </c>
+      <c r="H140" s="2" t="inlineStr">
+        <is>
+          <t>2756</t>
+        </is>
+      </c>
+      <c r="I140" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="J140" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="K140" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="L140" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="M140" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="N140" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="O140" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="P140" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="Q140" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="R140" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="S140" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="T140" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="U140" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="V140" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="W140" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="X140" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="Y140" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="Z140" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="AA140" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="AB140" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="AC140" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="AD140" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="AE140" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-09-07
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE140"/>
+  <dimension ref="A1:AE141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22452,6 +22452,163 @@
         </is>
       </c>
     </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>29098548792.328384</t>
+        </is>
+      </c>
+      <c r="C141" s="2" t="inlineStr">
+        <is>
+          <t>1995743122.9782412</t>
+        </is>
+      </c>
+      <c r="D141" s="2" t="inlineStr">
+        <is>
+          <t>80356</t>
+        </is>
+      </c>
+      <c r="E141" s="2" t="inlineStr">
+        <is>
+          <t>1995643952.658838</t>
+        </is>
+      </c>
+      <c r="F141" s="2" t="inlineStr">
+        <is>
+          <t>22825494227.090015</t>
+        </is>
+      </c>
+      <c r="G141" s="2" t="inlineStr">
+        <is>
+          <t>375545</t>
+        </is>
+      </c>
+      <c r="H141" s="2" t="inlineStr">
+        <is>
+          <t>3287</t>
+        </is>
+      </c>
+      <c r="I141" s="2" t="inlineStr">
+        <is>
+          <t>74116</t>
+        </is>
+      </c>
+      <c r="J141" s="2" t="inlineStr">
+        <is>
+          <t>343212</t>
+        </is>
+      </c>
+      <c r="K141" s="2" t="inlineStr">
+        <is>
+          <t>1022393</t>
+        </is>
+      </c>
+      <c r="L141" s="2" t="inlineStr">
+        <is>
+          <t>294.980000050407</t>
+        </is>
+      </c>
+      <c r="M141" s="2" t="inlineStr">
+        <is>
+          <t>65971.05533479631</t>
+        </is>
+      </c>
+      <c r="N141" s="2" t="inlineStr">
+        <is>
+          <t>262445.14933952945</t>
+        </is>
+      </c>
+      <c r="O141" s="2" t="inlineStr">
+        <is>
+          <t>880090.0326866627</t>
+        </is>
+      </c>
+      <c r="P141" s="2" t="inlineStr">
+        <is>
+          <t>10533.81</t>
+        </is>
+      </c>
+      <c r="Q141" s="2" t="inlineStr">
+        <is>
+          <t>404872723.39000005</t>
+        </is>
+      </c>
+      <c r="R141" s="2" t="inlineStr">
+        <is>
+          <t>1673315456.55</t>
+        </is>
+      </c>
+      <c r="S141" s="2" t="inlineStr">
+        <is>
+          <t>4912427456.4</t>
+        </is>
+      </c>
+      <c r="T141" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U141" s="2" t="inlineStr">
+        <is>
+          <t>4617</t>
+        </is>
+      </c>
+      <c r="V141" s="2" t="inlineStr">
+        <is>
+          <t>19025</t>
+        </is>
+      </c>
+      <c r="W141" s="2" t="inlineStr">
+        <is>
+          <t>56140</t>
+        </is>
+      </c>
+      <c r="X141" s="2" t="inlineStr">
+        <is>
+          <t>317796.67999999993</t>
+        </is>
+      </c>
+      <c r="Y141" s="2" t="inlineStr">
+        <is>
+          <t>116038206.19727556</t>
+        </is>
+      </c>
+      <c r="Z141" s="2" t="inlineStr">
+        <is>
+          <t>500067950.4772797</t>
+        </is>
+      </c>
+      <c r="AA141" s="2" t="inlineStr">
+        <is>
+          <t>1392429818.7681384</t>
+        </is>
+      </c>
+      <c r="AB141" s="2" t="inlineStr">
+        <is>
+          <t>107</t>
+        </is>
+      </c>
+      <c r="AC141" s="2" t="inlineStr">
+        <is>
+          <t>56502</t>
+        </is>
+      </c>
+      <c r="AD141" s="2" t="inlineStr">
+        <is>
+          <t>243510</t>
+        </is>
+      </c>
+      <c r="AE141" s="2" t="inlineStr">
+        <is>
+          <t>697462</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-09-08
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE141"/>
+  <dimension ref="A1:AE142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22609,6 +22609,163 @@
         </is>
       </c>
     </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>29102860595.67722</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>2002886399.1778212</t>
+        </is>
+      </c>
+      <c r="D142" s="2" t="inlineStr">
+        <is>
+          <t>80374</t>
+        </is>
+      </c>
+      <c r="E142" s="2" t="inlineStr">
+        <is>
+          <t>2002908199.0204563</t>
+        </is>
+      </c>
+      <c r="F142" s="2" t="inlineStr">
+        <is>
+          <t>22822040873.78</t>
+        </is>
+      </c>
+      <c r="G142" s="2" t="inlineStr">
+        <is>
+          <t>375555</t>
+        </is>
+      </c>
+      <c r="H142" s="2" t="inlineStr">
+        <is>
+          <t>2558</t>
+        </is>
+      </c>
+      <c r="I142" s="2" t="inlineStr">
+        <is>
+          <t>62825</t>
+        </is>
+      </c>
+      <c r="J142" s="2" t="inlineStr">
+        <is>
+          <t>343695</t>
+        </is>
+      </c>
+      <c r="K142" s="2" t="inlineStr">
+        <is>
+          <t>1012086</t>
+        </is>
+      </c>
+      <c r="L142" s="2" t="inlineStr">
+        <is>
+          <t>374.644666709341</t>
+        </is>
+      </c>
+      <c r="M142" s="2" t="inlineStr">
+        <is>
+          <t>57083.799001379164</t>
+        </is>
+      </c>
+      <c r="N142" s="2" t="inlineStr">
+        <is>
+          <t>259732.25033947593</t>
+        </is>
+      </c>
+      <c r="O142" s="2" t="inlineStr">
+        <is>
+          <t>869468.2223531206</t>
+        </is>
+      </c>
+      <c r="P142" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Q142" s="2" t="inlineStr">
+        <is>
+          <t>402359511.01000005</t>
+        </is>
+      </c>
+      <c r="R142" s="2" t="inlineStr">
+        <is>
+          <t>1620153218.87</t>
+        </is>
+      </c>
+      <c r="S142" s="2" t="inlineStr">
+        <is>
+          <t>4791451301.799999</t>
+        </is>
+      </c>
+      <c r="T142" s="2" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="U142" s="2" t="inlineStr">
+        <is>
+          <t>4605</t>
+        </is>
+      </c>
+      <c r="V142" s="2" t="inlineStr">
+        <is>
+          <t>18418</t>
+        </is>
+      </c>
+      <c r="W142" s="2" t="inlineStr">
+        <is>
+          <t>54854</t>
+        </is>
+      </c>
+      <c r="X142" s="2" t="inlineStr">
+        <is>
+          <t>641120.7600000002</t>
+        </is>
+      </c>
+      <c r="Y142" s="2" t="inlineStr">
+        <is>
+          <t>105576461.49075769</t>
+        </is>
+      </c>
+      <c r="Z142" s="2" t="inlineStr">
+        <is>
+          <t>497579540.7972797</t>
+        </is>
+      </c>
+      <c r="AA142" s="2" t="inlineStr">
+        <is>
+          <t>1371237850.0281384</t>
+        </is>
+      </c>
+      <c r="AB142" s="2" t="inlineStr">
+        <is>
+          <t>181</t>
+        </is>
+      </c>
+      <c r="AC142" s="2" t="inlineStr">
+        <is>
+          <t>59957</t>
+        </is>
+      </c>
+      <c r="AD142" s="2" t="inlineStr">
+        <is>
+          <t>242377</t>
+        </is>
+      </c>
+      <c r="AE142" s="2" t="inlineStr">
+        <is>
+          <t>697197</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-09-09
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE142"/>
+  <dimension ref="A1:AE143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22766,6 +22766,163 @@
         </is>
       </c>
     </row>
+    <row r="143">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
+        <is>
+          <t>29280550178.107735</t>
+        </is>
+      </c>
+      <c r="C143" s="2" t="inlineStr">
+        <is>
+          <t>2015355999.779263</t>
+        </is>
+      </c>
+      <c r="D143" s="2" t="inlineStr">
+        <is>
+          <t>80405</t>
+        </is>
+      </c>
+      <c r="E143" s="2" t="inlineStr">
+        <is>
+          <t>2015027828.069047</t>
+        </is>
+      </c>
+      <c r="F143" s="2" t="inlineStr">
+        <is>
+          <t>22950827331.87</t>
+        </is>
+      </c>
+      <c r="G143" s="2" t="inlineStr">
+        <is>
+          <t>376900</t>
+        </is>
+      </c>
+      <c r="H143" s="2" t="inlineStr">
+        <is>
+          <t>11522</t>
+        </is>
+      </c>
+      <c r="I143" s="2" t="inlineStr">
+        <is>
+          <t>56272</t>
+        </is>
+      </c>
+      <c r="J143" s="2" t="inlineStr">
+        <is>
+          <t>345107</t>
+        </is>
+      </c>
+      <c r="K143" s="2" t="inlineStr">
+        <is>
+          <t>1005893</t>
+        </is>
+      </c>
+      <c r="L143" s="2" t="inlineStr">
+        <is>
+          <t>3014.860333475676</t>
+        </is>
+      </c>
+      <c r="M143" s="2" t="inlineStr">
+        <is>
+          <t>54122.26000124152</t>
+        </is>
+      </c>
+      <c r="N143" s="2" t="inlineStr">
+        <is>
+          <t>269311.773672915</t>
+        </is>
+      </c>
+      <c r="O143" s="2" t="inlineStr">
+        <is>
+          <t>867846.6876861703</t>
+        </is>
+      </c>
+      <c r="P143" s="2" t="inlineStr">
+        <is>
+          <t>135395600.72999993</t>
+        </is>
+      </c>
+      <c r="Q143" s="2" t="inlineStr">
+        <is>
+          <t>279027430.5700001</t>
+        </is>
+      </c>
+      <c r="R143" s="2" t="inlineStr">
+        <is>
+          <t>1620944240.72</t>
+        </is>
+      </c>
+      <c r="S143" s="2" t="inlineStr">
+        <is>
+          <t>4722767408.049999</t>
+        </is>
+      </c>
+      <c r="T143" s="2" t="inlineStr">
+        <is>
+          <t>1534</t>
+        </is>
+      </c>
+      <c r="U143" s="2" t="inlineStr">
+        <is>
+          <t>3146</t>
+        </is>
+      </c>
+      <c r="V143" s="2" t="inlineStr">
+        <is>
+          <t>18426</t>
+        </is>
+      </c>
+      <c r="W143" s="2" t="inlineStr">
+        <is>
+          <t>54079</t>
+        </is>
+      </c>
+      <c r="X143" s="2" t="inlineStr">
+        <is>
+          <t>1594154.0399999998</t>
+        </is>
+      </c>
+      <c r="Y143" s="2" t="inlineStr">
+        <is>
+          <t>89723977.6709428</t>
+        </is>
+      </c>
+      <c r="Z143" s="2" t="inlineStr">
+        <is>
+          <t>504942469.207465</t>
+        </is>
+      </c>
+      <c r="AA143" s="2" t="inlineStr">
+        <is>
+          <t>1366780228.7683237</t>
+        </is>
+      </c>
+      <c r="AB143" s="2" t="inlineStr">
+        <is>
+          <t>236</t>
+        </is>
+      </c>
+      <c r="AC143" s="2" t="inlineStr">
+        <is>
+          <t>57556</t>
+        </is>
+      </c>
+      <c r="AD143" s="2" t="inlineStr">
+        <is>
+          <t>243352</t>
+        </is>
+      </c>
+      <c r="AE143" s="2" t="inlineStr">
+        <is>
+          <t>698576</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-09-10
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE143"/>
+  <dimension ref="A1:AE144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22923,6 +22923,163 @@
         </is>
       </c>
     </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>29380411751.479916</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>2019348593.5018167</t>
+        </is>
+      </c>
+      <c r="D144" s="2" t="inlineStr">
+        <is>
+          <t>80435</t>
+        </is>
+      </c>
+      <c r="E144" s="2" t="inlineStr">
+        <is>
+          <t>2019118681.8322518</t>
+        </is>
+      </c>
+      <c r="F144" s="2" t="inlineStr">
+        <is>
+          <t>23044412792.349987</t>
+        </is>
+      </c>
+      <c r="G144" s="2" t="inlineStr">
+        <is>
+          <t>378161</t>
+        </is>
+      </c>
+      <c r="H144" s="2" t="inlineStr">
+        <is>
+          <t>7413</t>
+        </is>
+      </c>
+      <c r="I144" s="2" t="inlineStr">
+        <is>
+          <t>61233</t>
+        </is>
+      </c>
+      <c r="J144" s="2" t="inlineStr">
+        <is>
+          <t>347474</t>
+        </is>
+      </c>
+      <c r="K144" s="2" t="inlineStr">
+        <is>
+          <t>1012705</t>
+        </is>
+      </c>
+      <c r="L144" s="2" t="inlineStr">
+        <is>
+          <t>2403.800000105434</t>
+        </is>
+      </c>
+      <c r="M144" s="2" t="inlineStr">
+        <is>
+          <t>56240.17766795524</t>
+        </is>
+      </c>
+      <c r="N144" s="2" t="inlineStr">
+        <is>
+          <t>274952.53333979455</t>
+        </is>
+      </c>
+      <c r="O144" s="2" t="inlineStr">
+        <is>
+          <t>868311.3470194123</t>
+        </is>
+      </c>
+      <c r="P144" s="2" t="inlineStr">
+        <is>
+          <t>72091396.8526</t>
+        </is>
+      </c>
+      <c r="Q144" s="2" t="inlineStr">
+        <is>
+          <t>337885270.7300002</t>
+        </is>
+      </c>
+      <c r="R144" s="2" t="inlineStr">
+        <is>
+          <t>1755889421.4</t>
+        </is>
+      </c>
+      <c r="S144" s="2" t="inlineStr">
+        <is>
+          <t>4793725160.66</t>
+        </is>
+      </c>
+      <c r="T144" s="2" t="inlineStr">
+        <is>
+          <t>791</t>
+        </is>
+      </c>
+      <c r="U144" s="2" t="inlineStr">
+        <is>
+          <t>3831</t>
+        </is>
+      </c>
+      <c r="V144" s="2" t="inlineStr">
+        <is>
+          <t>19967</t>
+        </is>
+      </c>
+      <c r="W144" s="2" t="inlineStr">
+        <is>
+          <t>54878</t>
+        </is>
+      </c>
+      <c r="X144" s="2" t="inlineStr">
+        <is>
+          <t>1822635.509999999</t>
+        </is>
+      </c>
+      <c r="Y144" s="2" t="inlineStr">
+        <is>
+          <t>90312023.0651481</t>
+        </is>
+      </c>
+      <c r="Z144" s="2" t="inlineStr">
+        <is>
+          <t>501201490.3116702</t>
+        </is>
+      </c>
+      <c r="AA144" s="2" t="inlineStr">
+        <is>
+          <t>1363772981.632529</t>
+        </is>
+      </c>
+      <c r="AB144" s="2" t="inlineStr">
+        <is>
+          <t>325</t>
+        </is>
+      </c>
+      <c r="AC144" s="2" t="inlineStr">
+        <is>
+          <t>56867</t>
+        </is>
+      </c>
+      <c r="AD144" s="2" t="inlineStr">
+        <is>
+          <t>243659</t>
+        </is>
+      </c>
+      <c r="AE144" s="2" t="inlineStr">
+        <is>
+          <t>699846</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-09-11
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE144"/>
+  <dimension ref="A1:AE145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23080,6 +23080,163 @@
         </is>
       </c>
     </row>
+    <row r="145">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B145" s="2" t="inlineStr">
+        <is>
+          <t>29523400223.670265</t>
+        </is>
+      </c>
+      <c r="C145" s="2" t="inlineStr">
+        <is>
+          <t>2034324305.594805</t>
+        </is>
+      </c>
+      <c r="D145" s="2" t="inlineStr">
+        <is>
+          <t>80457</t>
+        </is>
+      </c>
+      <c r="E145" s="2" t="inlineStr">
+        <is>
+          <t>2034032272.565621</t>
+        </is>
+      </c>
+      <c r="F145" s="2" t="inlineStr">
+        <is>
+          <t>23133438339.809994</t>
+        </is>
+      </c>
+      <c r="G145" s="2" t="inlineStr">
+        <is>
+          <t>379136</t>
+        </is>
+      </c>
+      <c r="H145" s="2" t="inlineStr">
+        <is>
+          <t>8214</t>
+        </is>
+      </c>
+      <c r="I145" s="2" t="inlineStr">
+        <is>
+          <t>63269</t>
+        </is>
+      </c>
+      <c r="J145" s="2" t="inlineStr">
+        <is>
+          <t>348201</t>
+        </is>
+      </c>
+      <c r="K145" s="2" t="inlineStr">
+        <is>
+          <t>1020268</t>
+        </is>
+      </c>
+      <c r="L145" s="2" t="inlineStr">
+        <is>
+          <t>2810.960000129512</t>
+        </is>
+      </c>
+      <c r="M145" s="2" t="inlineStr">
+        <is>
+          <t>59278.89900136471</t>
+        </is>
+      </c>
+      <c r="N145" s="2" t="inlineStr">
+        <is>
+          <t>275916.7840064445</t>
+        </is>
+      </c>
+      <c r="O145" s="2" t="inlineStr">
+        <is>
+          <t>869508.5083527723</t>
+        </is>
+      </c>
+      <c r="P145" s="2" t="inlineStr">
+        <is>
+          <t>78456127.11</t>
+        </is>
+      </c>
+      <c r="Q145" s="2" t="inlineStr">
+        <is>
+          <t>326391405.2638002</t>
+        </is>
+      </c>
+      <c r="R145" s="2" t="inlineStr">
+        <is>
+          <t>1702962659.0738003</t>
+        </is>
+      </c>
+      <c r="S145" s="2" t="inlineStr">
+        <is>
+          <t>4814633409.0138</t>
+        </is>
+      </c>
+      <c r="T145" s="2" t="inlineStr">
+        <is>
+          <t>887</t>
+        </is>
+      </c>
+      <c r="U145" s="2" t="inlineStr">
+        <is>
+          <t>3685</t>
+        </is>
+      </c>
+      <c r="V145" s="2" t="inlineStr">
+        <is>
+          <t>19303</t>
+        </is>
+      </c>
+      <c r="W145" s="2" t="inlineStr">
+        <is>
+          <t>55063</t>
+        </is>
+      </c>
+      <c r="X145" s="2" t="inlineStr">
+        <is>
+          <t>1682953.7599999998</t>
+        </is>
+      </c>
+      <c r="Y145" s="2" t="inlineStr">
+        <is>
+          <t>92459764.98439047</t>
+        </is>
+      </c>
+      <c r="Z145" s="2" t="inlineStr">
+        <is>
+          <t>497655144.6616701</t>
+        </is>
+      </c>
+      <c r="AA145" s="2" t="inlineStr">
+        <is>
+          <t>1359311927.0855298</t>
+        </is>
+      </c>
+      <c r="AB145" s="2" t="inlineStr">
+        <is>
+          <t>320</t>
+        </is>
+      </c>
+      <c r="AC145" s="2" t="inlineStr">
+        <is>
+          <t>57153</t>
+        </is>
+      </c>
+      <c r="AD145" s="2" t="inlineStr">
+        <is>
+          <t>246014</t>
+        </is>
+      </c>
+      <c r="AE145" s="2" t="inlineStr">
+        <is>
+          <t>701453</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-09-12
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE145"/>
+  <dimension ref="A1:AE146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23237,6 +23237,163 @@
         </is>
       </c>
     </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>29598888446.1288</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>2039517048.3585598</t>
+        </is>
+      </c>
+      <c r="D146" s="2" t="inlineStr">
+        <is>
+          <t>80474</t>
+        </is>
+      </c>
+      <c r="E146" s="2" t="inlineStr">
+        <is>
+          <t>2039475065.991484</t>
+        </is>
+      </c>
+      <c r="F146" s="2" t="inlineStr">
+        <is>
+          <t>23184149818.279995</t>
+        </is>
+      </c>
+      <c r="G146" s="2" t="inlineStr">
+        <is>
+          <t>379750</t>
+        </is>
+      </c>
+      <c r="H146" s="2" t="inlineStr">
+        <is>
+          <t>6967</t>
+        </is>
+      </c>
+      <c r="I146" s="2" t="inlineStr">
+        <is>
+          <t>69682</t>
+        </is>
+      </c>
+      <c r="J146" s="2" t="inlineStr">
+        <is>
+          <t>349961</t>
+        </is>
+      </c>
+      <c r="K146" s="2" t="inlineStr">
+        <is>
+          <t>1031720</t>
+        </is>
+      </c>
+      <c r="L146" s="2" t="inlineStr">
+        <is>
+          <t>2306.63200009584</t>
+        </is>
+      </c>
+      <c r="M146" s="2" t="inlineStr">
+        <is>
+          <t>59903.187001442144</t>
+        </is>
+      </c>
+      <c r="N146" s="2" t="inlineStr">
+        <is>
+          <t>277808.51467312954</t>
+        </is>
+      </c>
+      <c r="O146" s="2" t="inlineStr">
+        <is>
+          <t>878289.0296862695</t>
+        </is>
+      </c>
+      <c r="P146" s="2" t="inlineStr">
+        <is>
+          <t>55433646.08000003</t>
+        </is>
+      </c>
+      <c r="Q146" s="2" t="inlineStr">
+        <is>
+          <t>353862253.6238002</t>
+        </is>
+      </c>
+      <c r="R146" s="2" t="inlineStr">
+        <is>
+          <t>1702848975.7738004</t>
+        </is>
+      </c>
+      <c r="S146" s="2" t="inlineStr">
+        <is>
+          <t>4844130117.753799</t>
+        </is>
+      </c>
+      <c r="T146" s="2" t="inlineStr">
+        <is>
+          <t>632</t>
+        </is>
+      </c>
+      <c r="U146" s="2" t="inlineStr">
+        <is>
+          <t>3953</t>
+        </is>
+      </c>
+      <c r="V146" s="2" t="inlineStr">
+        <is>
+          <t>19284</t>
+        </is>
+      </c>
+      <c r="W146" s="2" t="inlineStr">
+        <is>
+          <t>55372</t>
+        </is>
+      </c>
+      <c r="X146" s="2" t="inlineStr">
+        <is>
+          <t>312003.57000000007</t>
+        </is>
+      </c>
+      <c r="Y146" s="2" t="inlineStr">
+        <is>
+          <t>99147530.18439043</t>
+        </is>
+      </c>
+      <c r="Z146" s="2" t="inlineStr">
+        <is>
+          <t>506454093.06167</t>
+        </is>
+      </c>
+      <c r="AA146" s="2" t="inlineStr">
+        <is>
+          <t>1373808774.5655296</t>
+        </is>
+      </c>
+      <c r="AB146" s="2" t="inlineStr">
+        <is>
+          <t>212</t>
+        </is>
+      </c>
+      <c r="AC146" s="2" t="inlineStr">
+        <is>
+          <t>57420</t>
+        </is>
+      </c>
+      <c r="AD146" s="2" t="inlineStr">
+        <is>
+          <t>247442</t>
+        </is>
+      </c>
+      <c r="AE146" s="2" t="inlineStr">
+        <is>
+          <t>703658</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-09-13
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE146"/>
+  <dimension ref="A1:AE147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23394,6 +23394,163 @@
         </is>
       </c>
     </row>
+    <row r="147">
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="inlineStr">
+        <is>
+          <t>29566526613.801125</t>
+        </is>
+      </c>
+      <c r="C147" s="2" t="inlineStr">
+        <is>
+          <t>2037151685.74041</t>
+        </is>
+      </c>
+      <c r="D147" s="2" t="inlineStr">
+        <is>
+          <t>80487</t>
+        </is>
+      </c>
+      <c r="E147" s="2" t="inlineStr">
+        <is>
+          <t>2037015336.5273201</t>
+        </is>
+      </c>
+      <c r="F147" s="2" t="inlineStr">
+        <is>
+          <t>23178654176.51</t>
+        </is>
+      </c>
+      <c r="G147" s="2" t="inlineStr">
+        <is>
+          <t>379693</t>
+        </is>
+      </c>
+      <c r="H147" s="2" t="inlineStr">
+        <is>
+          <t>3852</t>
+        </is>
+      </c>
+      <c r="I147" s="2" t="inlineStr">
+        <is>
+          <t>74463</t>
+        </is>
+      </c>
+      <c r="J147" s="2" t="inlineStr">
+        <is>
+          <t>341560</t>
+        </is>
+      </c>
+      <c r="K147" s="2" t="inlineStr">
+        <is>
+          <t>1032097</t>
+        </is>
+      </c>
+      <c r="L147" s="2" t="inlineStr">
+        <is>
+          <t>358.682333391291</t>
+        </is>
+      </c>
+      <c r="M147" s="2" t="inlineStr">
+        <is>
+          <t>59729.73433475485</t>
+        </is>
+      </c>
+      <c r="N147" s="2" t="inlineStr">
+        <is>
+          <t>272642.6523397124</t>
+        </is>
+      </c>
+      <c r="O147" s="2" t="inlineStr">
+        <is>
+          <t>880099.1423529864</t>
+        </is>
+      </c>
+      <c r="P147" s="2" t="inlineStr">
+        <is>
+          <t>114986.88</t>
+        </is>
+      </c>
+      <c r="Q147" s="2" t="inlineStr">
+        <is>
+          <t>348439780.59380025</t>
+        </is>
+      </c>
+      <c r="R147" s="2" t="inlineStr">
+        <is>
+          <t>1677603250.1038003</t>
+        </is>
+      </c>
+      <c r="S147" s="2" t="inlineStr">
+        <is>
+          <t>4899561417.3538</t>
+        </is>
+      </c>
+      <c r="T147" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="U147" s="2" t="inlineStr">
+        <is>
+          <t>3890</t>
+        </is>
+      </c>
+      <c r="V147" s="2" t="inlineStr">
+        <is>
+          <t>19034</t>
+        </is>
+      </c>
+      <c r="W147" s="2" t="inlineStr">
+        <is>
+          <t>56004</t>
+        </is>
+      </c>
+      <c r="X147" s="2" t="inlineStr">
+        <is>
+          <t>286831.09000000014</t>
+        </is>
+      </c>
+      <c r="Y147" s="2" t="inlineStr">
+        <is>
+          <t>99826965.35439047</t>
+        </is>
+      </c>
+      <c r="Z147" s="2" t="inlineStr">
+        <is>
+          <t>492705432.60167</t>
+        </is>
+      </c>
+      <c r="AA147" s="2" t="inlineStr">
+        <is>
+          <t>1376295265.8355296</t>
+        </is>
+      </c>
+      <c r="AB147" s="2" t="inlineStr">
+        <is>
+          <t>122</t>
+        </is>
+      </c>
+      <c r="AC147" s="2" t="inlineStr">
+        <is>
+          <t>57597</t>
+        </is>
+      </c>
+      <c r="AD147" s="2" t="inlineStr">
+        <is>
+          <t>247286</t>
+        </is>
+      </c>
+      <c r="AE147" s="2" t="inlineStr">
+        <is>
+          <t>704998</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-09-14
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE147"/>
+  <dimension ref="A1:AE148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23551,6 +23551,163 @@
         </is>
       </c>
     </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>29576454703.98013</t>
+        </is>
+      </c>
+      <c r="C148" s="2" t="inlineStr">
+        <is>
+          <t>2052785293.4738975</t>
+        </is>
+      </c>
+      <c r="D148" s="2" t="inlineStr">
+        <is>
+          <t>80506</t>
+        </is>
+      </c>
+      <c r="E148" s="2" t="inlineStr">
+        <is>
+          <t>2049153749.7219646</t>
+        </is>
+      </c>
+      <c r="F148" s="2" t="inlineStr">
+        <is>
+          <t>23175624539.280003</t>
+        </is>
+      </c>
+      <c r="G148" s="2" t="inlineStr">
+        <is>
+          <t>379662</t>
+        </is>
+      </c>
+      <c r="H148" s="2" t="inlineStr">
+        <is>
+          <t>3592</t>
+        </is>
+      </c>
+      <c r="I148" s="2" t="inlineStr">
+        <is>
+          <t>75035</t>
+        </is>
+      </c>
+      <c r="J148" s="2" t="inlineStr">
+        <is>
+          <t>338016</t>
+        </is>
+      </c>
+      <c r="K148" s="2" t="inlineStr">
+        <is>
+          <t>1021309</t>
+        </is>
+      </c>
+      <c r="L148" s="2" t="inlineStr">
+        <is>
+          <t>353.327333391515</t>
+        </is>
+      </c>
+      <c r="M148" s="2" t="inlineStr">
+        <is>
+          <t>60316.9760014422</t>
+        </is>
+      </c>
+      <c r="N148" s="2" t="inlineStr">
+        <is>
+          <t>265029.1653395678</t>
+        </is>
+      </c>
+      <c r="O148" s="2" t="inlineStr">
+        <is>
+          <t>872693.9206862209</t>
+        </is>
+      </c>
+      <c r="P148" s="2" t="inlineStr">
+        <is>
+          <t>5638.59</t>
+        </is>
+      </c>
+      <c r="Q148" s="2" t="inlineStr">
+        <is>
+          <t>348495882.79380023</t>
+        </is>
+      </c>
+      <c r="R148" s="2" t="inlineStr">
+        <is>
+          <t>1619532764.0338004</t>
+        </is>
+      </c>
+      <c r="S148" s="2" t="inlineStr">
+        <is>
+          <t>4899574113.0738</t>
+        </is>
+      </c>
+      <c r="T148" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U148" s="2" t="inlineStr">
+        <is>
+          <t>3892</t>
+        </is>
+      </c>
+      <c r="V148" s="2" t="inlineStr">
+        <is>
+          <t>18359</t>
+        </is>
+      </c>
+      <c r="W148" s="2" t="inlineStr">
+        <is>
+          <t>56003</t>
+        </is>
+      </c>
+      <c r="X148" s="2" t="inlineStr">
+        <is>
+          <t>1459986.9700000018</t>
+        </is>
+      </c>
+      <c r="Y148" s="2" t="inlineStr">
+        <is>
+          <t>98638213.84439048</t>
+        </is>
+      </c>
+      <c r="Z148" s="2" t="inlineStr">
+        <is>
+          <t>480092318.76167005</t>
+        </is>
+      </c>
+      <c r="AA148" s="2" t="inlineStr">
+        <is>
+          <t>1370289427.9455297</t>
+        </is>
+      </c>
+      <c r="AB148" s="2" t="inlineStr">
+        <is>
+          <t>1423</t>
+        </is>
+      </c>
+      <c r="AC148" s="2" t="inlineStr">
+        <is>
+          <t>57452</t>
+        </is>
+      </c>
+      <c r="AD148" s="2" t="inlineStr">
+        <is>
+          <t>246465</t>
+        </is>
+      </c>
+      <c r="AE148" s="2" t="inlineStr">
+        <is>
+          <t>704412</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-09-15
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE148"/>
+  <dimension ref="A1:AE149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23708,6 +23708,163 @@
         </is>
       </c>
     </row>
+    <row r="149">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B149" s="2" t="inlineStr">
+        <is>
+          <t>29721860747.700954</t>
+        </is>
+      </c>
+      <c r="C149" s="2" t="inlineStr">
+        <is>
+          <t>2053960456.8903887</t>
+        </is>
+      </c>
+      <c r="D149" s="2" t="inlineStr">
+        <is>
+          <t>80531</t>
+        </is>
+      </c>
+      <c r="E149" s="2" t="inlineStr">
+        <is>
+          <t>2051905978.3348699</t>
+        </is>
+      </c>
+      <c r="F149" s="2" t="inlineStr">
+        <is>
+          <t>23304690566.569996</t>
+        </is>
+      </c>
+      <c r="G149" s="2" t="inlineStr">
+        <is>
+          <t>381221</t>
+        </is>
+      </c>
+      <c r="H149" s="2" t="inlineStr">
+        <is>
+          <t>9850</t>
+        </is>
+      </c>
+      <c r="I149" s="2" t="inlineStr">
+        <is>
+          <t>76201</t>
+        </is>
+      </c>
+      <c r="J149" s="2" t="inlineStr">
+        <is>
+          <t>343246</t>
+        </is>
+      </c>
+      <c r="K149" s="2" t="inlineStr">
+        <is>
+          <t>1015616</t>
+        </is>
+      </c>
+      <c r="L149" s="2" t="inlineStr">
+        <is>
+          <t>2038.402333452002</t>
+        </is>
+      </c>
+      <c r="M149" s="2" t="inlineStr">
+        <is>
+          <t>69863.41966822227</t>
+        </is>
+      </c>
+      <c r="N149" s="2" t="inlineStr">
+        <is>
+          <t>271655.1660062582</t>
+        </is>
+      </c>
+      <c r="O149" s="2" t="inlineStr">
+        <is>
+          <t>871086.4066861499</t>
+        </is>
+      </c>
+      <c r="P149" s="2" t="inlineStr">
+        <is>
+          <t>120718576.48999995</t>
+        </is>
+      </c>
+      <c r="Q149" s="2" t="inlineStr">
+        <is>
+          <t>350720111.83380026</t>
+        </is>
+      </c>
+      <c r="R149" s="2" t="inlineStr">
+        <is>
+          <t>1557412811.1238005</t>
+        </is>
+      </c>
+      <c r="S149" s="2" t="inlineStr">
+        <is>
+          <t>4802602126.6838</t>
+        </is>
+      </c>
+      <c r="T149" s="2" t="inlineStr">
+        <is>
+          <t>1417</t>
+        </is>
+      </c>
+      <c r="U149" s="2" t="inlineStr">
+        <is>
+          <t>3907</t>
+        </is>
+      </c>
+      <c r="V149" s="2" t="inlineStr">
+        <is>
+          <t>17661</t>
+        </is>
+      </c>
+      <c r="W149" s="2" t="inlineStr">
+        <is>
+          <t>54900</t>
+        </is>
+      </c>
+      <c r="X149" s="2" t="inlineStr">
+        <is>
+          <t>1848503.1900000002</t>
+        </is>
+      </c>
+      <c r="Y149" s="2" t="inlineStr">
+        <is>
+          <t>107855455.54439047</t>
+        </is>
+      </c>
+      <c r="Z149" s="2" t="inlineStr">
+        <is>
+          <t>484885831.72167003</t>
+        </is>
+      </c>
+      <c r="AA149" s="2" t="inlineStr">
+        <is>
+          <t>1373675328.6555297</t>
+        </is>
+      </c>
+      <c r="AB149" s="2" t="inlineStr">
+        <is>
+          <t>260</t>
+        </is>
+      </c>
+      <c r="AC149" s="2" t="inlineStr">
+        <is>
+          <t>58713</t>
+        </is>
+      </c>
+      <c r="AD149" s="2" t="inlineStr">
+        <is>
+          <t>245139</t>
+        </is>
+      </c>
+      <c r="AE149" s="2" t="inlineStr">
+        <is>
+          <t>705126</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-09-16
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE149"/>
+  <dimension ref="A1:AE150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23865,6 +23865,163 @@
         </is>
       </c>
     </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>29847073458.68766</t>
+        </is>
+      </c>
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>2055924020.8744626</t>
+        </is>
+      </c>
+      <c r="D150" s="2" t="inlineStr">
+        <is>
+          <t>80550</t>
+        </is>
+      </c>
+      <c r="E150" s="2" t="inlineStr">
+        <is>
+          <t>2055497088.0975187</t>
+        </is>
+      </c>
+      <c r="F150" s="2" t="inlineStr">
+        <is>
+          <t>23402790799.66</t>
+        </is>
+      </c>
+      <c r="G150" s="2" t="inlineStr">
+        <is>
+          <t>382348</t>
+        </is>
+      </c>
+      <c r="H150" s="2" t="inlineStr">
+        <is>
+          <t>10899</t>
+        </is>
+      </c>
+      <c r="I150" s="2" t="inlineStr">
+        <is>
+          <t>74911</t>
+        </is>
+      </c>
+      <c r="J150" s="2" t="inlineStr">
+        <is>
+          <t>354224</t>
+        </is>
+      </c>
+      <c r="K150" s="2" t="inlineStr">
+        <is>
+          <t>1020524</t>
+        </is>
+      </c>
+      <c r="L150" s="2" t="inlineStr">
+        <is>
+          <t>3238.286333473793</t>
+        </is>
+      </c>
+      <c r="M150" s="2" t="inlineStr">
+        <is>
+          <t>72250.62266837529</t>
+        </is>
+      </c>
+      <c r="N150" s="2" t="inlineStr">
+        <is>
+          <t>283557.5343398384</t>
+        </is>
+      </c>
+      <c r="O150" s="2" t="inlineStr">
+        <is>
+          <t>873463.2333528674</t>
+        </is>
+      </c>
+      <c r="P150" s="2" t="inlineStr">
+        <is>
+          <t>95293821.12000006</t>
+        </is>
+      </c>
+      <c r="Q150" s="2" t="inlineStr">
+        <is>
+          <t>472363471.8838002</t>
+        </is>
+      </c>
+      <c r="R150" s="2" t="inlineStr">
+        <is>
+          <t>1679847193.0238004</t>
+        </is>
+      </c>
+      <c r="S150" s="2" t="inlineStr">
+        <is>
+          <t>4857468136.0638</t>
+        </is>
+      </c>
+      <c r="T150" s="2" t="inlineStr">
+        <is>
+          <t>1003</t>
+        </is>
+      </c>
+      <c r="U150" s="2" t="inlineStr">
+        <is>
+          <t>5326</t>
+        </is>
+      </c>
+      <c r="V150" s="2" t="inlineStr">
+        <is>
+          <t>19088</t>
+        </is>
+      </c>
+      <c r="W150" s="2" t="inlineStr">
+        <is>
+          <t>55541</t>
+        </is>
+      </c>
+      <c r="X150" s="2" t="inlineStr">
+        <is>
+          <t>1859906.3200000008</t>
+        </is>
+      </c>
+      <c r="Y150" s="2" t="inlineStr">
+        <is>
+          <t>111323241.12420519</t>
+        </is>
+      </c>
+      <c r="Z150" s="2" t="inlineStr">
+        <is>
+          <t>496915744.51167005</t>
+        </is>
+      </c>
+      <c r="AA150" s="2" t="inlineStr">
+        <is>
+          <t>1380285270.2655296</t>
+        </is>
+      </c>
+      <c r="AB150" s="2" t="inlineStr">
+        <is>
+          <t>304</t>
+        </is>
+      </c>
+      <c r="AC150" s="2" t="inlineStr">
+        <is>
+          <t>60359</t>
+        </is>
+      </c>
+      <c r="AD150" s="2" t="inlineStr">
+        <is>
+          <t>247629</t>
+        </is>
+      </c>
+      <c r="AE150" s="2" t="inlineStr">
+        <is>
+          <t>707076</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-09-17
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE150"/>
+  <dimension ref="A1:AE151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24022,6 +24022,163 @@
         </is>
       </c>
     </row>
+    <row r="151">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B151" s="2" t="inlineStr">
+        <is>
+          <t>29952562236.29943</t>
+        </is>
+      </c>
+      <c r="C151" s="2" t="inlineStr">
+        <is>
+          <t>2066924149.741531</t>
+        </is>
+      </c>
+      <c r="D151" s="2" t="inlineStr">
+        <is>
+          <t>80572</t>
+        </is>
+      </c>
+      <c r="E151" s="2" t="inlineStr">
+        <is>
+          <t>2066160311.24658</t>
+        </is>
+      </c>
+      <c r="F151" s="2" t="inlineStr">
+        <is>
+          <t>23487328591.58001</t>
+        </is>
+      </c>
+      <c r="G151" s="2" t="inlineStr">
+        <is>
+          <t>383364</t>
+        </is>
+      </c>
+      <c r="H151" s="2" t="inlineStr">
+        <is>
+          <t>8996</t>
+        </is>
+      </c>
+      <c r="I151" s="2" t="inlineStr">
+        <is>
+          <t>77128</t>
+        </is>
+      </c>
+      <c r="J151" s="2" t="inlineStr">
+        <is>
+          <t>355304</t>
+        </is>
+      </c>
+      <c r="K151" s="2" t="inlineStr">
+        <is>
+          <t>1028440</t>
+        </is>
+      </c>
+      <c r="L151" s="2" t="inlineStr">
+        <is>
+          <t>2457.611333449755</t>
+        </is>
+      </c>
+      <c r="M151" s="2" t="inlineStr">
+        <is>
+          <t>71839.64800168622</t>
+        </is>
+      </c>
+      <c r="N151" s="2" t="inlineStr">
+        <is>
+          <t>286081.1290066415</t>
+        </is>
+      </c>
+      <c r="O151" s="2" t="inlineStr">
+        <is>
+          <t>874023.5266861576</t>
+        </is>
+      </c>
+      <c r="P151" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q151" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R151" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S151" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T151" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U151" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V151" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W151" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X151" s="2" t="inlineStr">
+        <is>
+          <t>1237635.3599999999</t>
+        </is>
+      </c>
+      <c r="Y151" s="2" t="inlineStr">
+        <is>
+          <t>114641780.27999982</t>
+        </is>
+      </c>
+      <c r="Z151" s="2" t="inlineStr">
+        <is>
+          <t>499549635.95167</t>
+        </is>
+      </c>
+      <c r="AA151" s="2" t="inlineStr">
+        <is>
+          <t>1388808887.8004556</t>
+        </is>
+      </c>
+      <c r="AB151" s="2" t="inlineStr">
+        <is>
+          <t>280</t>
+        </is>
+      </c>
+      <c r="AC151" s="2" t="inlineStr">
+        <is>
+          <t>60637</t>
+        </is>
+      </c>
+      <c r="AD151" s="2" t="inlineStr">
+        <is>
+          <t>247052</t>
+        </is>
+      </c>
+      <c r="AE151" s="2" t="inlineStr">
+        <is>
+          <t>707187</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-09-18
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE151"/>
+  <dimension ref="A1:AE152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24179,6 +24179,163 @@
         </is>
       </c>
     </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>30068581331.11718</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="inlineStr">
+        <is>
+          <t>2094975676.2494774</t>
+        </is>
+      </c>
+      <c r="D152" s="2" t="inlineStr">
+        <is>
+          <t>80586</t>
+        </is>
+      </c>
+      <c r="E152" s="2" t="inlineStr">
+        <is>
+          <t>2092436134.4347153</t>
+        </is>
+      </c>
+      <c r="F152" s="2" t="inlineStr">
+        <is>
+          <t>23551497550.809994</t>
+        </is>
+      </c>
+      <c r="G152" s="2" t="inlineStr">
+        <is>
+          <t>384014</t>
+        </is>
+      </c>
+      <c r="H152" s="2" t="inlineStr">
+        <is>
+          <t>8242</t>
+        </is>
+      </c>
+      <c r="I152" s="2" t="inlineStr">
+        <is>
+          <t>75478</t>
+        </is>
+      </c>
+      <c r="J152" s="2" t="inlineStr">
+        <is>
+          <t>353559</t>
+        </is>
+      </c>
+      <c r="K152" s="2" t="inlineStr">
+        <is>
+          <t>1038474</t>
+        </is>
+      </c>
+      <c r="L152" s="2" t="inlineStr">
+        <is>
+          <t>2081.198000142366</t>
+        </is>
+      </c>
+      <c r="M152" s="2" t="inlineStr">
+        <is>
+          <t>69442.67733491218</t>
+        </is>
+      </c>
+      <c r="N152" s="2" t="inlineStr">
+        <is>
+          <t>283526.5370065631</t>
+        </is>
+      </c>
+      <c r="O152" s="2" t="inlineStr">
+        <is>
+          <t>879033.8173527718</t>
+        </is>
+      </c>
+      <c r="P152" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q152" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R152" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S152" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T152" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U152" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V152" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W152" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X152" s="2" t="inlineStr">
+        <is>
+          <t>1677320.5800000003</t>
+        </is>
+      </c>
+      <c r="Y152" s="2" t="inlineStr">
+        <is>
+          <t>120913539.92999999</t>
+        </is>
+      </c>
+      <c r="Z152" s="2" t="inlineStr">
+        <is>
+          <t>501159338.2416701</t>
+        </is>
+      </c>
+      <c r="AA152" s="2" t="inlineStr">
+        <is>
+          <t>1403915376.8104556</t>
+        </is>
+      </c>
+      <c r="AB152" s="2" t="inlineStr">
+        <is>
+          <t>282</t>
+        </is>
+      </c>
+      <c r="AC152" s="2" t="inlineStr">
+        <is>
+          <t>61909</t>
+        </is>
+      </c>
+      <c r="AD152" s="2" t="inlineStr">
+        <is>
+          <t>249471</t>
+        </is>
+      </c>
+      <c r="AE152" s="2" t="inlineStr">
+        <is>
+          <t>711764</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-09-19
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE152"/>
+  <dimension ref="A1:AE153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24336,6 +24336,163 @@
         </is>
       </c>
     </row>
+    <row r="153">
+      <c r="A153" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B153" s="2" t="inlineStr">
+        <is>
+          <t>30184107255.213444</t>
+        </is>
+      </c>
+      <c r="C153" s="2" t="inlineStr">
+        <is>
+          <t>2110721977.420199</t>
+        </is>
+      </c>
+      <c r="D153" s="2" t="inlineStr">
+        <is>
+          <t>80608</t>
+        </is>
+      </c>
+      <c r="E153" s="2" t="inlineStr">
+        <is>
+          <t>2110620739.224743</t>
+        </is>
+      </c>
+      <c r="F153" s="2" t="inlineStr">
+        <is>
+          <t>23636003567.979992</t>
+        </is>
+      </c>
+      <c r="G153" s="2" t="inlineStr">
+        <is>
+          <t>384906</t>
+        </is>
+      </c>
+      <c r="H153" s="2" t="inlineStr">
+        <is>
+          <t>7835</t>
+        </is>
+      </c>
+      <c r="I153" s="2" t="inlineStr">
+        <is>
+          <t>80278</t>
+        </is>
+      </c>
+      <c r="J153" s="2" t="inlineStr">
+        <is>
+          <t>352642</t>
+        </is>
+      </c>
+      <c r="K153" s="2" t="inlineStr">
+        <is>
+          <t>1048552</t>
+        </is>
+      </c>
+      <c r="L153" s="2" t="inlineStr">
+        <is>
+          <t>1747.956000109319</t>
+        </is>
+      </c>
+      <c r="M153" s="2" t="inlineStr">
+        <is>
+          <t>67115.43066815482</t>
+        </is>
+      </c>
+      <c r="N153" s="2" t="inlineStr">
+        <is>
+          <t>282217.7970064654</t>
+        </is>
+      </c>
+      <c r="O153" s="2" t="inlineStr">
+        <is>
+          <t>886503.9133529231</t>
+        </is>
+      </c>
+      <c r="P153" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q153" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R153" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S153" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T153" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U153" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V153" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W153" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X153" s="2" t="inlineStr">
+        <is>
+          <t>1076465.2000000002</t>
+        </is>
+      </c>
+      <c r="Y153" s="2" t="inlineStr">
+        <is>
+          <t>117103667.17000008</t>
+        </is>
+      </c>
+      <c r="Z153" s="2" t="inlineStr">
+        <is>
+          <t>501129728.3816701</t>
+        </is>
+      </c>
+      <c r="AA153" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="AB153" s="2" t="inlineStr">
+        <is>
+          <t>228</t>
+        </is>
+      </c>
+      <c r="AC153" s="2" t="inlineStr">
+        <is>
+          <t>62864</t>
+        </is>
+      </c>
+      <c r="AD153" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="AE153" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-09-20
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE153"/>
+  <dimension ref="A1:AE154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24493,6 +24493,163 @@
         </is>
       </c>
     </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>30182392092.045372</t>
+        </is>
+      </c>
+      <c r="C154" s="2" t="inlineStr">
+        <is>
+          <t>2113829465.3887796</t>
+        </is>
+      </c>
+      <c r="D154" s="2" t="inlineStr">
+        <is>
+          <t>80619</t>
+        </is>
+      </c>
+      <c r="E154" s="2" t="inlineStr">
+        <is>
+          <t>2113028453.4703596</t>
+        </is>
+      </c>
+      <c r="F154" s="2" t="inlineStr">
+        <is>
+          <t>23632821623.429996</t>
+        </is>
+      </c>
+      <c r="G154" s="2" t="inlineStr">
+        <is>
+          <t>384774</t>
+        </is>
+      </c>
+      <c r="H154" s="2" t="inlineStr">
+        <is>
+          <t>3028</t>
+        </is>
+      </c>
+      <c r="I154" s="2" t="inlineStr">
+        <is>
+          <t>85645</t>
+        </is>
+      </c>
+      <c r="J154" s="2" t="inlineStr">
+        <is>
+          <t>348837</t>
+        </is>
+      </c>
+      <c r="K154" s="2" t="inlineStr">
+        <is>
+          <t>1051283</t>
+        </is>
+      </c>
+      <c r="L154" s="2" t="inlineStr">
+        <is>
+          <t>329.56466670813</t>
+        </is>
+      </c>
+      <c r="M154" s="2" t="inlineStr">
+        <is>
+          <t>66691.08366819298</t>
+        </is>
+      </c>
+      <c r="N154" s="2" t="inlineStr">
+        <is>
+          <t>274222.4746730433</t>
+        </is>
+      </c>
+      <c r="O154" s="2" t="inlineStr">
+        <is>
+          <t>887926.34801968</t>
+        </is>
+      </c>
+      <c r="P154" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q154" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R154" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S154" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T154" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U154" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V154" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W154" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X154" s="2" t="inlineStr">
+        <is>
+          <t>536686.14</t>
+        </is>
+      </c>
+      <c r="Y154" s="2" t="inlineStr">
+        <is>
+          <t>114557820.48000003</t>
+        </is>
+      </c>
+      <c r="Z154" s="2" t="inlineStr">
+        <is>
+          <t>483090904.60469824</t>
+        </is>
+      </c>
+      <c r="AA154" s="2" t="inlineStr">
+        <is>
+          <t>1416162259.9104555</t>
+        </is>
+      </c>
+      <c r="AB154" s="2" t="inlineStr">
+        <is>
+          <t>123</t>
+        </is>
+      </c>
+      <c r="AC154" s="2" t="inlineStr">
+        <is>
+          <t>61459</t>
+        </is>
+      </c>
+      <c r="AD154" s="2" t="inlineStr">
+        <is>
+          <t>249488</t>
+        </is>
+      </c>
+      <c r="AE154" s="2" t="inlineStr">
+        <is>
+          <t>714509</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-09-21
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE154"/>
+  <dimension ref="A1:AE155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24650,6 +24650,163 @@
         </is>
       </c>
     </row>
+    <row r="155">
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B155" s="2" t="inlineStr">
+        <is>
+          <t>30184524996.70905</t>
+        </is>
+      </c>
+      <c r="C155" s="2" t="inlineStr">
+        <is>
+          <t>2120688010.9458907</t>
+        </is>
+      </c>
+      <c r="D155" s="2" t="inlineStr">
+        <is>
+          <t>80640</t>
+        </is>
+      </c>
+      <c r="E155" s="2" t="inlineStr">
+        <is>
+          <t>2118352002.9561887</t>
+        </is>
+      </c>
+      <c r="F155" s="2" t="inlineStr">
+        <is>
+          <t>23629472221.56001</t>
+        </is>
+      </c>
+      <c r="G155" s="2" t="inlineStr">
+        <is>
+          <t>384728</t>
+        </is>
+      </c>
+      <c r="H155" s="2" t="inlineStr">
+        <is>
+          <t>3781</t>
+        </is>
+      </c>
+      <c r="I155" s="2" t="inlineStr">
+        <is>
+          <t>80488</t>
+        </is>
+      </c>
+      <c r="J155" s="2" t="inlineStr">
+        <is>
+          <t>344264</t>
+        </is>
+      </c>
+      <c r="K155" s="2" t="inlineStr">
+        <is>
+          <t>1039384</t>
+        </is>
+      </c>
+      <c r="L155" s="2" t="inlineStr">
+        <is>
+          <t>443.380000066297</t>
+        </is>
+      </c>
+      <c r="M155" s="2" t="inlineStr">
+        <is>
+          <t>66496.66566817004</t>
+        </is>
+      </c>
+      <c r="N155" s="2" t="inlineStr">
+        <is>
+          <t>264635.010006175</t>
+        </is>
+      </c>
+      <c r="O155" s="2" t="inlineStr">
+        <is>
+          <t>880896.4493529253</t>
+        </is>
+      </c>
+      <c r="P155" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q155" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R155" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S155" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T155" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U155" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V155" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W155" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X155" s="2" t="inlineStr">
+        <is>
+          <t>418513.6100000002</t>
+        </is>
+      </c>
+      <c r="Y155" s="2" t="inlineStr">
+        <is>
+          <t>115792054.03000005</t>
+        </is>
+      </c>
+      <c r="Z155" s="2" t="inlineStr">
+        <is>
+          <t>473884406.97469825</t>
+        </is>
+      </c>
+      <c r="AA155" s="2" t="inlineStr">
+        <is>
+          <t>1414526196.3504555</t>
+        </is>
+      </c>
+      <c r="AB155" s="2" t="inlineStr">
+        <is>
+          <t>157</t>
+        </is>
+      </c>
+      <c r="AC155" s="2" t="inlineStr">
+        <is>
+          <t>62401</t>
+        </is>
+      </c>
+      <c r="AD155" s="2" t="inlineStr">
+        <is>
+          <t>250154</t>
+        </is>
+      </c>
+      <c r="AE155" s="2" t="inlineStr">
+        <is>
+          <t>715882</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-09-22
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE155"/>
+  <dimension ref="A1:AE156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24807,6 +24807,163 @@
         </is>
       </c>
     </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>30371015710.33783</t>
+        </is>
+      </c>
+      <c r="C156" s="2" t="inlineStr">
+        <is>
+          <t>2125064497.8811681</t>
+        </is>
+      </c>
+      <c r="D156" s="2" t="inlineStr">
+        <is>
+          <t>80663</t>
+        </is>
+      </c>
+      <c r="E156" s="2" t="inlineStr">
+        <is>
+          <t>2124814747.700178</t>
+        </is>
+      </c>
+      <c r="F156" s="2" t="inlineStr">
+        <is>
+          <t>23780008923.280006</t>
+        </is>
+      </c>
+      <c r="G156" s="2" t="inlineStr">
+        <is>
+          <t>386422</t>
+        </is>
+      </c>
+      <c r="H156" s="2" t="inlineStr">
+        <is>
+          <t>11781</t>
+        </is>
+      </c>
+      <c r="I156" s="2" t="inlineStr">
+        <is>
+          <t>70280</t>
+        </is>
+      </c>
+      <c r="J156" s="2" t="inlineStr">
+        <is>
+          <t>348375</t>
+        </is>
+      </c>
+      <c r="K156" s="2" t="inlineStr">
+        <is>
+          <t>1031960</t>
+        </is>
+      </c>
+      <c r="L156" s="2" t="inlineStr">
+        <is>
+          <t>3238.981666831911</t>
+        </is>
+      </c>
+      <c r="M156" s="2" t="inlineStr">
+        <is>
+          <t>66193.75233480647</t>
+        </is>
+      </c>
+      <c r="N156" s="2" t="inlineStr">
+        <is>
+          <t>271024.8920061714</t>
+        </is>
+      </c>
+      <c r="O156" s="2" t="inlineStr">
+        <is>
+          <t>874545.4893527222</t>
+        </is>
+      </c>
+      <c r="P156" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q156" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R156" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S156" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T156" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U156" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V156" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W156" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X156" s="2" t="inlineStr">
+        <is>
+          <t>963455.3799999999</t>
+        </is>
+      </c>
+      <c r="Y156" s="2" t="inlineStr">
+        <is>
+          <t>111151235.66999999</t>
+        </is>
+      </c>
+      <c r="Z156" s="2" t="inlineStr">
+        <is>
+          <t>475859943.8146981</t>
+        </is>
+      </c>
+      <c r="AA156" s="2" t="inlineStr">
+        <is>
+          <t>1405236208.269904</t>
+        </is>
+      </c>
+      <c r="AB156" s="2" t="inlineStr">
+        <is>
+          <t>221</t>
+        </is>
+      </c>
+      <c r="AC156" s="2" t="inlineStr">
+        <is>
+          <t>62168</t>
+        </is>
+      </c>
+      <c r="AD156" s="2" t="inlineStr">
+        <is>
+          <t>249563</t>
+        </is>
+      </c>
+      <c r="AE156" s="2" t="inlineStr">
+        <is>
+          <t>716049</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-09-23
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE156"/>
+  <dimension ref="A1:AE157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24964,6 +24964,163 @@
         </is>
       </c>
     </row>
+    <row r="157">
+      <c r="A157" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B157" s="2" t="inlineStr">
+        <is>
+          <t>30474387947.545097</t>
+        </is>
+      </c>
+      <c r="C157" s="2" t="inlineStr">
+        <is>
+          <t>2129833794.617944</t>
+        </is>
+      </c>
+      <c r="D157" s="2" t="inlineStr">
+        <is>
+          <t>80688</t>
+        </is>
+      </c>
+      <c r="E157" s="2" t="inlineStr">
+        <is>
+          <t>2129543418.6849618</t>
+        </is>
+      </c>
+      <c r="F157" s="2" t="inlineStr">
+        <is>
+          <t>23867155971.740005</t>
+        </is>
+      </c>
+      <c r="G157" s="2" t="inlineStr">
+        <is>
+          <t>387411</t>
+        </is>
+      </c>
+      <c r="H157" s="2" t="inlineStr">
+        <is>
+          <t>9016</t>
+        </is>
+      </c>
+      <c r="I157" s="2" t="inlineStr">
+        <is>
+          <t>70616</t>
+        </is>
+      </c>
+      <c r="J157" s="2" t="inlineStr">
+        <is>
+          <t>357150</t>
+        </is>
+      </c>
+      <c r="K157" s="2" t="inlineStr">
+        <is>
+          <t>1030365</t>
+        </is>
+      </c>
+      <c r="L157" s="2" t="inlineStr">
+        <is>
+          <t>2376.063666808601</t>
+        </is>
+      </c>
+      <c r="M157" s="2" t="inlineStr">
+        <is>
+          <t>65245.936001441376</t>
+        </is>
+      </c>
+      <c r="N157" s="2" t="inlineStr">
+        <is>
+          <t>281389.92100637895</t>
+        </is>
+      </c>
+      <c r="O157" s="2" t="inlineStr">
+        <is>
+          <t>872295.3400192983</t>
+        </is>
+      </c>
+      <c r="P157" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q157" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R157" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S157" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T157" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U157" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V157" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W157" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X157" s="2" t="inlineStr">
+        <is>
+          <t>1116382.9800000002</t>
+        </is>
+      </c>
+      <c r="Y157" s="2" t="inlineStr">
+        <is>
+          <t>113505457.17999999</t>
+        </is>
+      </c>
+      <c r="Z157" s="2" t="inlineStr">
+        <is>
+          <t>489883230.5346981</t>
+        </is>
+      </c>
+      <c r="AA157" s="2" t="inlineStr">
+        <is>
+          <t>1410374715.219904</t>
+        </is>
+      </c>
+      <c r="AB157" s="2" t="inlineStr">
+        <is>
+          <t>223</t>
+        </is>
+      </c>
+      <c r="AC157" s="2" t="inlineStr">
+        <is>
+          <t>60855</t>
+        </is>
+      </c>
+      <c r="AD157" s="2" t="inlineStr">
+        <is>
+          <t>250553</t>
+        </is>
+      </c>
+      <c r="AE157" s="2" t="inlineStr">
+        <is>
+          <t>717269</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-09-24
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE157"/>
+  <dimension ref="A1:AE158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25121,6 +25121,163 @@
         </is>
       </c>
     </row>
+    <row r="158">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B158" s="2" t="inlineStr">
+        <is>
+          <t>30538389829.089127</t>
+        </is>
+      </c>
+      <c r="C158" s="2" t="inlineStr">
+        <is>
+          <t>2180016398.437366</t>
+        </is>
+      </c>
+      <c r="D158" s="2" t="inlineStr">
+        <is>
+          <t>80718</t>
+        </is>
+      </c>
+      <c r="E158" s="2" t="inlineStr">
+        <is>
+          <t>2168460569.918318</t>
+        </is>
+      </c>
+      <c r="F158" s="2" t="inlineStr">
+        <is>
+          <t>23951412963.809994</t>
+        </is>
+      </c>
+      <c r="G158" s="2" t="inlineStr">
+        <is>
+          <t>388268</t>
+        </is>
+      </c>
+      <c r="H158" s="2" t="inlineStr">
+        <is>
+          <t>9398</t>
+        </is>
+      </c>
+      <c r="I158" s="2" t="inlineStr">
+        <is>
+          <t>72816</t>
+        </is>
+      </c>
+      <c r="J158" s="2" t="inlineStr">
+        <is>
+          <t>355719</t>
+        </is>
+      </c>
+      <c r="K158" s="2" t="inlineStr">
+        <is>
+          <t>1032833</t>
+        </is>
+      </c>
+      <c r="L158" s="2" t="inlineStr">
+        <is>
+          <t>1265.188000085196</t>
+        </is>
+      </c>
+      <c r="M158" s="2" t="inlineStr">
+        <is>
+          <t>64819.78300142555</t>
+        </is>
+      </c>
+      <c r="N158" s="2" t="inlineStr">
+        <is>
+          <t>282832.73600643064</t>
+        </is>
+      </c>
+      <c r="O158" s="2" t="inlineStr">
+        <is>
+          <t>870894.1476857873</t>
+        </is>
+      </c>
+      <c r="P158" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q158" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R158" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S158" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T158" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U158" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V158" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W158" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X158" s="2" t="inlineStr">
+        <is>
+          <t>1058541.5999999996</t>
+        </is>
+      </c>
+      <c r="Y158" s="2" t="inlineStr">
+        <is>
+          <t>111750366.36000012</t>
+        </is>
+      </c>
+      <c r="Z158" s="2" t="inlineStr">
+        <is>
+          <t>487389353.7246983</t>
+        </is>
+      </c>
+      <c r="AA158" s="2" t="inlineStr">
+        <is>
+          <t>1416480428.659904</t>
+        </is>
+      </c>
+      <c r="AB158" s="2" t="inlineStr">
+        <is>
+          <t>264</t>
+        </is>
+      </c>
+      <c r="AC158" s="2" t="inlineStr">
+        <is>
+          <t>60963</t>
+        </is>
+      </c>
+      <c r="AD158" s="2" t="inlineStr">
+        <is>
+          <t>250487</t>
+        </is>
+      </c>
+      <c r="AE158" s="2" t="inlineStr">
+        <is>
+          <t>719350</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-09-25
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE158"/>
+  <dimension ref="A1:AE159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25278,6 +25278,163 @@
         </is>
       </c>
     </row>
+    <row r="159">
+      <c r="A159" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B159" s="2" t="inlineStr">
+        <is>
+          <t>30709395962.43473</t>
+        </is>
+      </c>
+      <c r="C159" s="2" t="inlineStr">
+        <is>
+          <t>2185871452.325978</t>
+        </is>
+      </c>
+      <c r="D159" s="2" t="inlineStr">
+        <is>
+          <t>80746</t>
+        </is>
+      </c>
+      <c r="E159" s="2" t="inlineStr">
+        <is>
+          <t>2185465437.449867</t>
+        </is>
+      </c>
+      <c r="F159" s="2" t="inlineStr">
+        <is>
+          <t>24016906914.77001</t>
+        </is>
+      </c>
+      <c r="G159" s="2" t="inlineStr">
+        <is>
+          <t>388959</t>
+        </is>
+      </c>
+      <c r="H159" s="2" t="inlineStr">
+        <is>
+          <t>9365</t>
+        </is>
+      </c>
+      <c r="I159" s="2" t="inlineStr">
+        <is>
+          <t>74088</t>
+        </is>
+      </c>
+      <c r="J159" s="2" t="inlineStr">
+        <is>
+          <t>355864</t>
+        </is>
+      </c>
+      <c r="K159" s="2" t="inlineStr">
+        <is>
+          <t>1039567</t>
+        </is>
+      </c>
+      <c r="L159" s="2" t="inlineStr">
+        <is>
+          <t>2322.366666785879</t>
+        </is>
+      </c>
+      <c r="M159" s="2" t="inlineStr">
+        <is>
+          <t>62600.07833478473</t>
+        </is>
+      </c>
+      <c r="N159" s="2" t="inlineStr">
+        <is>
+          <t>277449.96467301715</t>
+        </is>
+      </c>
+      <c r="O159" s="2" t="inlineStr">
+        <is>
+          <t>868497.5306857367</t>
+        </is>
+      </c>
+      <c r="P159" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q159" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R159" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S159" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T159" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U159" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V159" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W159" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X159" s="2" t="inlineStr">
+        <is>
+          <t>1255494.2500000002</t>
+        </is>
+      </c>
+      <c r="Y159" s="2" t="inlineStr">
+        <is>
+          <t>109399445.27999987</t>
+        </is>
+      </c>
+      <c r="Z159" s="2" t="inlineStr">
+        <is>
+          <t>489407755.2546981</t>
+        </is>
+      </c>
+      <c r="AA159" s="2" t="inlineStr">
+        <is>
+          <t>1400354253.3099039</t>
+        </is>
+      </c>
+      <c r="AB159" s="2" t="inlineStr">
+        <is>
+          <t>306</t>
+        </is>
+      </c>
+      <c r="AC159" s="2" t="inlineStr">
+        <is>
+          <t>60369</t>
+        </is>
+      </c>
+      <c r="AD159" s="2" t="inlineStr">
+        <is>
+          <t>253842</t>
+        </is>
+      </c>
+      <c r="AE159" s="2" t="inlineStr">
+        <is>
+          <t>721145</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-09-26
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE159"/>
+  <dimension ref="A1:AE160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25435,6 +25435,163 @@
         </is>
       </c>
     </row>
+    <row r="160">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B160" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="C160" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="D160" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="E160" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="F160" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="G160" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="H160" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="I160" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="J160" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="K160" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="L160" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="M160" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="N160" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="O160" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="P160" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="Q160" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="R160" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="S160" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="T160" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="U160" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="V160" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="W160" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="X160" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="Y160" s="2" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="Z160" s="2" t="inlineStr">
+        <is>
+          <t>490921651.024698</t>
+        </is>
+      </c>
+      <c r="AA160" s="2" t="inlineStr">
+        <is>
+          <t>1415490789.4899037</t>
+        </is>
+      </c>
+      <c r="AB160" s="2" t="inlineStr">
+        <is>
+          <t>226</t>
+        </is>
+      </c>
+      <c r="AC160" s="2" t="inlineStr">
+        <is>
+          <t>59188</t>
+        </is>
+      </c>
+      <c r="AD160" s="2" t="inlineStr">
+        <is>
+          <t>254425</t>
+        </is>
+      </c>
+      <c r="AE160" s="2" t="inlineStr">
+        <is>
+          <t>722441</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-09-27
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE160"/>
+  <dimension ref="A1:AE161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25592,6 +25592,163 @@
         </is>
       </c>
     </row>
+    <row r="161">
+      <c r="A161" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B161" s="2" t="inlineStr">
+        <is>
+          <t>30825042981.469704</t>
+        </is>
+      </c>
+      <c r="C161" s="2" t="inlineStr">
+        <is>
+          <t>2202573891.0165706</t>
+        </is>
+      </c>
+      <c r="D161" s="2" t="inlineStr">
+        <is>
+          <t>80777</t>
+        </is>
+      </c>
+      <c r="E161" s="2" t="inlineStr">
+        <is>
+          <t>2201137976.6446705</t>
+        </is>
+      </c>
+      <c r="F161" s="2" t="inlineStr">
+        <is>
+          <t>24094009248.890007</t>
+        </is>
+      </c>
+      <c r="G161" s="2" t="inlineStr">
+        <is>
+          <t>389629</t>
+        </is>
+      </c>
+      <c r="H161" s="2" t="inlineStr">
+        <is>
+          <t>3685</t>
+        </is>
+      </c>
+      <c r="I161" s="2" t="inlineStr">
+        <is>
+          <t>85497</t>
+        </is>
+      </c>
+      <c r="J161" s="2" t="inlineStr">
+        <is>
+          <t>353244</t>
+        </is>
+      </c>
+      <c r="K161" s="2" t="inlineStr">
+        <is>
+          <t>1052737</t>
+        </is>
+      </c>
+      <c r="L161" s="2" t="inlineStr">
+        <is>
+          <t>311.670333393048</t>
+        </is>
+      </c>
+      <c r="M161" s="2" t="inlineStr">
+        <is>
+          <t>61801.79900140935</t>
+        </is>
+      </c>
+      <c r="N161" s="2" t="inlineStr">
+        <is>
+          <t>269164.7270062219</t>
+        </is>
+      </c>
+      <c r="O161" s="2" t="inlineStr">
+        <is>
+          <t>875809.916019199</t>
+        </is>
+      </c>
+      <c r="P161" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q161" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R161" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S161" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T161" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U161" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V161" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W161" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X161" s="2" t="inlineStr">
+        <is>
+          <t>4170697.97999999</t>
+        </is>
+      </c>
+      <c r="Y161" s="2" t="inlineStr">
+        <is>
+          <t>117171495.89843512</t>
+        </is>
+      </c>
+      <c r="Z161" s="2" t="inlineStr">
+        <is>
+          <t>475303380.9431334</t>
+        </is>
+      </c>
+      <c r="AA161" s="2" t="inlineStr">
+        <is>
+          <t>1415636243.5183392</t>
+        </is>
+      </c>
+      <c r="AB161" s="2" t="inlineStr">
+        <is>
+          <t>5026</t>
+        </is>
+      </c>
+      <c r="AC161" s="2" t="inlineStr">
+        <is>
+          <t>60946</t>
+        </is>
+      </c>
+      <c r="AD161" s="2" t="inlineStr">
+        <is>
+          <t>252866</t>
+        </is>
+      </c>
+      <c r="AE161" s="2" t="inlineStr">
+        <is>
+          <t>722912</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-09-28
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE161"/>
+  <dimension ref="A1:AE162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25749,6 +25749,163 @@
         </is>
       </c>
     </row>
+    <row r="162">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B162" s="2" t="inlineStr">
+        <is>
+          <t>30814624189.6026</t>
+        </is>
+      </c>
+      <c r="C162" s="2" t="inlineStr">
+        <is>
+          <t>2221748552.02784</t>
+        </is>
+      </c>
+      <c r="D162" s="2" t="inlineStr">
+        <is>
+          <t>80800</t>
+        </is>
+      </c>
+      <c r="E162" s="2" t="inlineStr">
+        <is>
+          <t>2215899388.9328065</t>
+        </is>
+      </c>
+      <c r="F162" s="2" t="inlineStr">
+        <is>
+          <t>24090013959.16</t>
+        </is>
+      </c>
+      <c r="G162" s="2" t="inlineStr">
+        <is>
+          <t>389587</t>
+        </is>
+      </c>
+      <c r="H162" s="2" t="inlineStr">
+        <is>
+          <t>3770</t>
+        </is>
+      </c>
+      <c r="I162" s="2" t="inlineStr">
+        <is>
+          <t>81402</t>
+        </is>
+      </c>
+      <c r="J162" s="2" t="inlineStr">
+        <is>
+          <t>349030</t>
+        </is>
+      </c>
+      <c r="K162" s="2" t="inlineStr">
+        <is>
+          <t>1044078</t>
+        </is>
+      </c>
+      <c r="L162" s="2" t="inlineStr">
+        <is>
+          <t>333.614000053626</t>
+        </is>
+      </c>
+      <c r="M162" s="2" t="inlineStr">
+        <is>
+          <t>61399.669668069895</t>
+        </is>
+      </c>
+      <c r="N162" s="2" t="inlineStr">
+        <is>
+          <t>259668.12233935847</t>
+        </is>
+      </c>
+      <c r="O162" s="2" t="inlineStr">
+        <is>
+          <t>867139.7080190643</t>
+        </is>
+      </c>
+      <c r="P162" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q162" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R162" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S162" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T162" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U162" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V162" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W162" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X162" s="2" t="inlineStr">
+        <is>
+          <t>7755220.739999996</t>
+        </is>
+      </c>
+      <c r="Y162" s="2" t="inlineStr">
+        <is>
+          <t>117107957.76843509</t>
+        </is>
+      </c>
+      <c r="Z162" s="2" t="inlineStr">
+        <is>
+          <t>464328556.5951012</t>
+        </is>
+      </c>
+      <c r="AA162" s="2" t="inlineStr">
+        <is>
+          <t>1411338674.4183393</t>
+        </is>
+      </c>
+      <c r="AB162" s="2" t="inlineStr">
+        <is>
+          <t>8077</t>
+        </is>
+      </c>
+      <c r="AC162" s="2" t="inlineStr">
+        <is>
+          <t>60707</t>
+        </is>
+      </c>
+      <c r="AD162" s="2" t="inlineStr">
+        <is>
+          <t>251597</t>
+        </is>
+      </c>
+      <c r="AE162" s="2" t="inlineStr">
+        <is>
+          <t>725223</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-09-29
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE162"/>
+  <dimension ref="A1:AE163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25906,6 +25906,163 @@
         </is>
       </c>
     </row>
+    <row r="163">
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B163" s="2" t="inlineStr">
+        <is>
+          <t>30952935153.116863</t>
+        </is>
+      </c>
+      <c r="C163" s="2" t="inlineStr">
+        <is>
+          <t>2219316877.072841</t>
+        </is>
+      </c>
+      <c r="D163" s="2" t="inlineStr">
+        <is>
+          <t>80820</t>
+        </is>
+      </c>
+      <c r="E163" s="2" t="inlineStr">
+        <is>
+          <t>2216687715.272601</t>
+        </is>
+      </c>
+      <c r="F163" s="2" t="inlineStr">
+        <is>
+          <t>24214633842.440002</t>
+        </is>
+      </c>
+      <c r="G163" s="2" t="inlineStr">
+        <is>
+          <t>391272</t>
+        </is>
+      </c>
+      <c r="H163" s="2" t="inlineStr">
+        <is>
+          <t>12394</t>
+        </is>
+      </c>
+      <c r="I163" s="2" t="inlineStr">
+        <is>
+          <t>72505</t>
+        </is>
+      </c>
+      <c r="J163" s="2" t="inlineStr">
+        <is>
+          <t>353717</t>
+        </is>
+      </c>
+      <c r="K163" s="2" t="inlineStr">
+        <is>
+          <t>1040231</t>
+        </is>
+      </c>
+      <c r="L163" s="2" t="inlineStr">
+        <is>
+          <t>2382.880000148106</t>
+        </is>
+      </c>
+      <c r="M163" s="2" t="inlineStr">
+        <is>
+          <t>59023.72366805752</t>
+        </is>
+      </c>
+      <c r="N163" s="2" t="inlineStr">
+        <is>
+          <t>264082.78767268965</t>
+        </is>
+      </c>
+      <c r="O163" s="2" t="inlineStr">
+        <is>
+          <t>861745.0070189801</t>
+        </is>
+      </c>
+      <c r="P163" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q163" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R163" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S163" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T163" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U163" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V163" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W163" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X163" s="2" t="inlineStr">
+        <is>
+          <t>996673.5799999997</t>
+        </is>
+      </c>
+      <c r="Y163" s="2" t="inlineStr">
+        <is>
+          <t>125926314.32843518</t>
+        </is>
+      </c>
+      <c r="Z163" s="2" t="inlineStr">
+        <is>
+          <t>475910873.86510116</t>
+        </is>
+      </c>
+      <c r="AA163" s="2" t="inlineStr">
+        <is>
+          <t>1405770607.418339</t>
+        </is>
+      </c>
+      <c r="AB163" s="2" t="inlineStr">
+        <is>
+          <t>254</t>
+        </is>
+      </c>
+      <c r="AC163" s="2" t="inlineStr">
+        <is>
+          <t>62284</t>
+        </is>
+      </c>
+      <c r="AD163" s="2" t="inlineStr">
+        <is>
+          <t>253543</t>
+        </is>
+      </c>
+      <c r="AE163" s="2" t="inlineStr">
+        <is>
+          <t>727095</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-09-30
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE163"/>
+  <dimension ref="A1:AE164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26063,6 +26063,163 @@
         </is>
       </c>
     </row>
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B164" s="2" t="inlineStr">
+        <is>
+          <t>31092050705.71868</t>
+        </is>
+      </c>
+      <c r="C164" s="2" t="inlineStr">
+        <is>
+          <t>2244238153.4568596</t>
+        </is>
+      </c>
+      <c r="D164" s="2" t="inlineStr">
+        <is>
+          <t>80837</t>
+        </is>
+      </c>
+      <c r="E164" s="2" t="inlineStr">
+        <is>
+          <t>2242546285.0449214</t>
+        </is>
+      </c>
+      <c r="F164" s="2" t="inlineStr">
+        <is>
+          <t>24283509669.280003</t>
+        </is>
+      </c>
+      <c r="G164" s="2" t="inlineStr">
+        <is>
+          <t>391712</t>
+        </is>
+      </c>
+      <c r="H164" s="2" t="inlineStr">
+        <is>
+          <t>6390</t>
+        </is>
+      </c>
+      <c r="I164" s="2" t="inlineStr">
+        <is>
+          <t>74046</t>
+        </is>
+      </c>
+      <c r="J164" s="2" t="inlineStr">
+        <is>
+          <t>361712</t>
+        </is>
+      </c>
+      <c r="K164" s="2" t="inlineStr">
+        <is>
+          <t>1038595</t>
+        </is>
+      </c>
+      <c r="L164" s="2" t="inlineStr">
+        <is>
+          <t>1458.818666756381</t>
+        </is>
+      </c>
+      <c r="M164" s="2" t="inlineStr">
+        <is>
+          <t>58421.24766804757</t>
+        </is>
+      </c>
+      <c r="N164" s="2" t="inlineStr">
+        <is>
+          <t>274572.7543395718</t>
+        </is>
+      </c>
+      <c r="O164" s="2" t="inlineStr">
+        <is>
+          <t>862914.8533523387</t>
+        </is>
+      </c>
+      <c r="P164" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q164" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R164" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S164" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T164" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U164" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V164" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W164" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X164" s="2" t="inlineStr">
+        <is>
+          <t>1013639.5899999999</t>
+        </is>
+      </c>
+      <c r="Y164" s="2" t="inlineStr">
+        <is>
+          <t>122699772.79843512</t>
+        </is>
+      </c>
+      <c r="Z164" s="2" t="inlineStr">
+        <is>
+          <t>486999902.77010113</t>
+        </is>
+      </c>
+      <c r="AA164" s="2" t="inlineStr">
+        <is>
+          <t>1401044733.4783392</t>
+        </is>
+      </c>
+      <c r="AB164" s="2" t="inlineStr">
+        <is>
+          <t>342</t>
+        </is>
+      </c>
+      <c r="AC164" s="2" t="inlineStr">
+        <is>
+          <t>61407</t>
+        </is>
+      </c>
+      <c r="AD164" s="2" t="inlineStr">
+        <is>
+          <t>254341</t>
+        </is>
+      </c>
+      <c r="AE164" s="2" t="inlineStr">
+        <is>
+          <t>724083</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-10-01
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE164"/>
+  <dimension ref="A1:AE165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26220,6 +26220,163 @@
         </is>
       </c>
     </row>
+    <row r="165">
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B165" s="2" t="inlineStr">
+        <is>
+          <t>31157018228.108337</t>
+        </is>
+      </c>
+      <c r="C165" s="2" t="inlineStr">
+        <is>
+          <t>2230874200.118438</t>
+        </is>
+      </c>
+      <c r="D165" s="2" t="inlineStr">
+        <is>
+          <t>80856</t>
+        </is>
+      </c>
+      <c r="E165" s="2" t="inlineStr">
+        <is>
+          <t>2230682336.527883</t>
+        </is>
+      </c>
+      <c r="F165" s="2" t="inlineStr">
+        <is>
+          <t>24362622863.280006</t>
+        </is>
+      </c>
+      <c r="G165" s="2" t="inlineStr">
+        <is>
+          <t>392256</t>
+        </is>
+      </c>
+      <c r="H165" s="2" t="inlineStr">
+        <is>
+          <t>7499</t>
+        </is>
+      </c>
+      <c r="I165" s="2" t="inlineStr">
+        <is>
+          <t>72692</t>
+        </is>
+      </c>
+      <c r="J165" s="2" t="inlineStr">
+        <is>
+          <t>359782</t>
+        </is>
+      </c>
+      <c r="K165" s="2" t="inlineStr">
+        <is>
+          <t>1042078</t>
+        </is>
+      </c>
+      <c r="L165" s="2" t="inlineStr">
+        <is>
+          <t>1179.630000095562</t>
+        </is>
+      </c>
+      <c r="M165" s="2" t="inlineStr">
+        <is>
+          <t>55863.124001299686</t>
+        </is>
+      </c>
+      <c r="N165" s="2" t="inlineStr">
+        <is>
+          <t>274040.97633960185</t>
+        </is>
+      </c>
+      <c r="O165" s="2" t="inlineStr">
+        <is>
+          <t>858275.2993521616</t>
+        </is>
+      </c>
+      <c r="P165" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q165" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R165" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S165" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T165" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U165" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V165" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W165" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X165" s="2" t="inlineStr">
+        <is>
+          <t>1751888.6599999997</t>
+        </is>
+      </c>
+      <c r="Y165" s="2" t="inlineStr">
+        <is>
+          <t>121448248.16194014</t>
+        </is>
+      </c>
+      <c r="Z165" s="2" t="inlineStr">
+        <is>
+          <t>487999806.50708836</t>
+        </is>
+      </c>
+      <c r="AA165" s="2" t="inlineStr">
+        <is>
+          <t>1398095093.7518442</t>
+        </is>
+      </c>
+      <c r="AB165" s="2" t="inlineStr">
+        <is>
+          <t>426</t>
+        </is>
+      </c>
+      <c r="AC165" s="2" t="inlineStr">
+        <is>
+          <t>62622</t>
+        </is>
+      </c>
+      <c r="AD165" s="2" t="inlineStr">
+        <is>
+          <t>260957</t>
+        </is>
+      </c>
+      <c r="AE165" s="2" t="inlineStr">
+        <is>
+          <t>724800</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-10-02
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE165"/>
+  <dimension ref="A1:AE166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26377,6 +26377,163 @@
         </is>
       </c>
     </row>
+    <row r="166">
+      <c r="A166" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B166" s="2" t="inlineStr">
+        <is>
+          <t>31305253576.493233</t>
+        </is>
+      </c>
+      <c r="C166" s="2" t="inlineStr">
+        <is>
+          <t>2336356908.698937</t>
+        </is>
+      </c>
+      <c r="D166" s="2" t="inlineStr">
+        <is>
+          <t>80884</t>
+        </is>
+      </c>
+      <c r="E166" s="2" t="inlineStr">
+        <is>
+          <t>2334486739.740538</t>
+        </is>
+      </c>
+      <c r="F166" s="2" t="inlineStr">
+        <is>
+          <t>24397733781.32999</t>
+        </is>
+      </c>
+      <c r="G166" s="2" t="inlineStr">
+        <is>
+          <t>393159</t>
+        </is>
+      </c>
+      <c r="H166" s="2" t="inlineStr">
+        <is>
+          <t>13307</t>
+        </is>
+      </c>
+      <c r="I166" s="2" t="inlineStr">
+        <is>
+          <t>69414</t>
+        </is>
+      </c>
+      <c r="J166" s="2" t="inlineStr">
+        <is>
+          <t>358383</t>
+        </is>
+      </c>
+      <c r="K166" s="2" t="inlineStr">
+        <is>
+          <t>1051143</t>
+        </is>
+      </c>
+      <c r="L166" s="2" t="inlineStr">
+        <is>
+          <t>2432.050000140065</t>
+        </is>
+      </c>
+      <c r="M166" s="2" t="inlineStr">
+        <is>
+          <t>52856.4130012207</t>
+        </is>
+      </c>
+      <c r="N166" s="2" t="inlineStr">
+        <is>
+          <t>266219.3713394526</t>
+        </is>
+      </c>
+      <c r="O166" s="2" t="inlineStr">
+        <is>
+          <t>857737.1913520794</t>
+        </is>
+      </c>
+      <c r="P166" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q166" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R166" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S166" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T166" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U166" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V166" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W166" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X166" s="2" t="inlineStr">
+        <is>
+          <t>1017188.9200000006</t>
+        </is>
+      </c>
+      <c r="Y166" s="2" t="inlineStr">
+        <is>
+          <t>125491964.85194042</t>
+        </is>
+      </c>
+      <c r="Z166" s="2" t="inlineStr">
+        <is>
+          <t>482182012.6070883</t>
+        </is>
+      </c>
+      <c r="AA166" s="2" t="inlineStr">
+        <is>
+          <t>1413881649.571844</t>
+        </is>
+      </c>
+      <c r="AB166" s="2" t="inlineStr">
+        <is>
+          <t>464</t>
+        </is>
+      </c>
+      <c r="AC166" s="2" t="inlineStr">
+        <is>
+          <t>65670</t>
+        </is>
+      </c>
+      <c r="AD166" s="2" t="inlineStr">
+        <is>
+          <t>263424</t>
+        </is>
+      </c>
+      <c r="AE166" s="2" t="inlineStr">
+        <is>
+          <t>730145</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-10-03
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE166"/>
+  <dimension ref="A1:AE167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26534,6 +26534,163 @@
         </is>
       </c>
     </row>
+    <row r="167">
+      <c r="A167" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B167" s="2" t="inlineStr">
+        <is>
+          <t>31413560619.291748</t>
+        </is>
+      </c>
+      <c r="C167" s="2" t="inlineStr">
+        <is>
+          <t>2322185860.4769616</t>
+        </is>
+      </c>
+      <c r="D167" s="2" t="inlineStr">
+        <is>
+          <t>80901</t>
+        </is>
+      </c>
+      <c r="E167" s="2" t="inlineStr">
+        <is>
+          <t>2326707195.426201</t>
+        </is>
+      </c>
+      <c r="F167" s="2" t="inlineStr">
+        <is>
+          <t>24500549017.280006</t>
+        </is>
+      </c>
+      <c r="G167" s="2" t="inlineStr">
+        <is>
+          <t>394060</t>
+        </is>
+      </c>
+      <c r="H167" s="2" t="inlineStr">
+        <is>
+          <t>9081</t>
+        </is>
+      </c>
+      <c r="I167" s="2" t="inlineStr">
+        <is>
+          <t>79560</t>
+        </is>
+      </c>
+      <c r="J167" s="2" t="inlineStr">
+        <is>
+          <t>362617</t>
+        </is>
+      </c>
+      <c r="K167" s="2" t="inlineStr">
+        <is>
+          <t>1067054</t>
+        </is>
+      </c>
+      <c r="L167" s="2" t="inlineStr">
+        <is>
+          <t>1189.718333435325</t>
+        </is>
+      </c>
+      <c r="M167" s="2" t="inlineStr">
+        <is>
+          <t>55124.73100122164</t>
+        </is>
+      </c>
+      <c r="N167" s="2" t="inlineStr">
+        <is>
+          <t>267650.8236727769</t>
+        </is>
+      </c>
+      <c r="O167" s="2" t="inlineStr">
+        <is>
+          <t>868645.9113522317</t>
+        </is>
+      </c>
+      <c r="P167" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q167" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R167" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S167" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T167" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U167" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V167" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W167" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X167" s="2" t="inlineStr">
+        <is>
+          <t>1283494.2200000002</t>
+        </is>
+      </c>
+      <c r="Y167" s="2" t="inlineStr">
+        <is>
+          <t>118784711.9119405</t>
+        </is>
+      </c>
+      <c r="Z167" s="2" t="inlineStr">
+        <is>
+          <t>482094197.0570883</t>
+        </is>
+      </c>
+      <c r="AA167" s="2" t="inlineStr">
+        <is>
+          <t>1425041600.3918443</t>
+        </is>
+      </c>
+      <c r="AB167" s="2" t="inlineStr">
+        <is>
+          <t>261</t>
+        </is>
+      </c>
+      <c r="AC167" s="2" t="inlineStr">
+        <is>
+          <t>67668</t>
+        </is>
+      </c>
+      <c r="AD167" s="2" t="inlineStr">
+        <is>
+          <t>265114</t>
+        </is>
+      </c>
+      <c r="AE167" s="2" t="inlineStr">
+        <is>
+          <t>734330</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-10-04
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE167"/>
+  <dimension ref="A1:AE168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26691,6 +26691,163 @@
         </is>
       </c>
     </row>
+    <row r="168">
+      <c r="A168" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B168" s="2" t="inlineStr">
+        <is>
+          <t>31440177370.53986</t>
+        </is>
+      </c>
+      <c r="C168" s="2" t="inlineStr">
+        <is>
+          <t>2332673038.380635</t>
+        </is>
+      </c>
+      <c r="D168" s="2" t="inlineStr">
+        <is>
+          <t>80915</t>
+        </is>
+      </c>
+      <c r="E168" s="2" t="inlineStr">
+        <is>
+          <t>2331130050.219175</t>
+        </is>
+      </c>
+      <c r="F168" s="2" t="inlineStr">
+        <is>
+          <t>24519466894.86001</t>
+        </is>
+      </c>
+      <c r="G168" s="2" t="inlineStr">
+        <is>
+          <t>394108</t>
+        </is>
+      </c>
+      <c r="H168" s="2" t="inlineStr">
+        <is>
+          <t>3803</t>
+        </is>
+      </c>
+      <c r="I168" s="2" t="inlineStr">
+        <is>
+          <t>85568</t>
+        </is>
+      </c>
+      <c r="J168" s="2" t="inlineStr">
+        <is>
+          <t>359804</t>
+        </is>
+      </c>
+      <c r="K168" s="2" t="inlineStr">
+        <is>
+          <t>1070434</t>
+        </is>
+      </c>
+      <c r="L168" s="2" t="inlineStr">
+        <is>
+          <t>213.73000004758</t>
+        </is>
+      </c>
+      <c r="M168" s="2" t="inlineStr">
+        <is>
+          <t>54042.31566788442</t>
+        </is>
+      </c>
+      <c r="N168" s="2" t="inlineStr">
+        <is>
+          <t>259950.42867266422</t>
+        </is>
+      </c>
+      <c r="O168" s="2" t="inlineStr">
+        <is>
+          <t>870164.4536856276</t>
+        </is>
+      </c>
+      <c r="P168" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q168" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R168" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S168" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T168" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U168" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V168" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W168" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X168" s="2" t="inlineStr">
+        <is>
+          <t>5787262.5399999805</t>
+        </is>
+      </c>
+      <c r="Y168" s="2" t="inlineStr">
+        <is>
+          <t>121694076.74350512</t>
+        </is>
+      </c>
+      <c r="Z168" s="2" t="inlineStr">
+        <is>
+          <t>477166033.6663307</t>
+        </is>
+      </c>
+      <c r="AA168" s="2" t="inlineStr">
+        <is>
+          <t>1429106577.0418441</t>
+        </is>
+      </c>
+      <c r="AB168" s="2" t="inlineStr">
+        <is>
+          <t>6944</t>
+        </is>
+      </c>
+      <c r="AC168" s="2" t="inlineStr">
+        <is>
+          <t>68597</t>
+        </is>
+      </c>
+      <c r="AD168" s="2" t="inlineStr">
+        <is>
+          <t>264676</t>
+        </is>
+      </c>
+      <c r="AE168" s="2" t="inlineStr">
+        <is>
+          <t>736526</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-10-05
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE168"/>
+  <dimension ref="A1:AE169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26848,6 +26848,163 @@
         </is>
       </c>
     </row>
+    <row r="169">
+      <c r="A169" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B169" s="2" t="inlineStr">
+        <is>
+          <t>31442809415.21117</t>
+        </is>
+      </c>
+      <c r="C169" s="2" t="inlineStr">
+        <is>
+          <t>2340725027.648298</t>
+        </is>
+      </c>
+      <c r="D169" s="2" t="inlineStr">
+        <is>
+          <t>80934</t>
+        </is>
+      </c>
+      <c r="E169" s="2" t="inlineStr">
+        <is>
+          <t>2337070086.570334</t>
+        </is>
+      </c>
+      <c r="F169" s="2" t="inlineStr">
+        <is>
+          <t>24516247820.63</t>
+        </is>
+      </c>
+      <c r="G169" s="2" t="inlineStr">
+        <is>
+          <t>394078</t>
+        </is>
+      </c>
+      <c r="H169" s="2" t="inlineStr">
+        <is>
+          <t>3497</t>
+        </is>
+      </c>
+      <c r="I169" s="2" t="inlineStr">
+        <is>
+          <t>81212</t>
+        </is>
+      </c>
+      <c r="J169" s="2" t="inlineStr">
+        <is>
+          <t>355083</t>
+        </is>
+      </c>
+      <c r="K169" s="2" t="inlineStr">
+        <is>
+          <t>1061085</t>
+        </is>
+      </c>
+      <c r="L169" s="2" t="inlineStr">
+        <is>
+          <t>304.80833337359</t>
+        </is>
+      </c>
+      <c r="M169" s="2" t="inlineStr">
+        <is>
+          <t>53630.33700121172</t>
+        </is>
+      </c>
+      <c r="N169" s="2" t="inlineStr">
+        <is>
+          <t>248201.36533912475</t>
+        </is>
+      </c>
+      <c r="O169" s="2" t="inlineStr">
+        <is>
+          <t>862245.6090188875</t>
+        </is>
+      </c>
+      <c r="P169" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q169" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R169" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S169" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T169" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U169" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V169" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W169" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X169" s="2" t="inlineStr">
+        <is>
+          <t>6117053.96000002</t>
+        </is>
+      </c>
+      <c r="Y169" s="2" t="inlineStr">
+        <is>
+          <t>120369439.1535051</t>
+        </is>
+      </c>
+      <c r="Z169" s="2" t="inlineStr">
+        <is>
+          <t>468867822.4063307</t>
+        </is>
+      </c>
+      <c r="AA169" s="2" t="inlineStr">
+        <is>
+          <t>1423850137.341844</t>
+        </is>
+      </c>
+      <c r="AB169" s="2" t="inlineStr">
+        <is>
+          <t>6709</t>
+        </is>
+      </c>
+      <c r="AC169" s="2" t="inlineStr">
+        <is>
+          <t>67650</t>
+        </is>
+      </c>
+      <c r="AD169" s="2" t="inlineStr">
+        <is>
+          <t>263549</t>
+        </is>
+      </c>
+      <c r="AE169" s="2" t="inlineStr">
+        <is>
+          <t>736527</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-10-06
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE169"/>
+  <dimension ref="A1:AE170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27005,6 +27005,163 @@
         </is>
       </c>
     </row>
+    <row r="170">
+      <c r="A170" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B170" s="2" t="inlineStr">
+        <is>
+          <t>31557274643.034195</t>
+        </is>
+      </c>
+      <c r="C170" s="2" t="inlineStr">
+        <is>
+          <t>2362208851.506717</t>
+        </is>
+      </c>
+      <c r="D170" s="2" t="inlineStr">
+        <is>
+          <t>80956</t>
+        </is>
+      </c>
+      <c r="E170" s="2" t="inlineStr">
+        <is>
+          <t>2346996450.817634</t>
+        </is>
+      </c>
+      <c r="F170" s="2" t="inlineStr">
+        <is>
+          <t>24626735668.88999</t>
+        </is>
+      </c>
+      <c r="G170" s="2" t="inlineStr">
+        <is>
+          <t>395684</t>
+        </is>
+      </c>
+      <c r="H170" s="2" t="inlineStr">
+        <is>
+          <t>13543</t>
+        </is>
+      </c>
+      <c r="I170" s="2" t="inlineStr">
+        <is>
+          <t>71219</t>
+        </is>
+      </c>
+      <c r="J170" s="2" t="inlineStr">
+        <is>
+          <t>358815</t>
+        </is>
+      </c>
+      <c r="K170" s="2" t="inlineStr">
+        <is>
+          <t>1056123</t>
+        </is>
+      </c>
+      <c r="L170" s="2" t="inlineStr">
+        <is>
+          <t>1857.89733345294</t>
+        </is>
+      </c>
+      <c r="M170" s="2" t="inlineStr">
+        <is>
+          <t>52122.881001156646</t>
+        </is>
+      </c>
+      <c r="N170" s="2" t="inlineStr">
+        <is>
+          <t>250133.49600571618</t>
+        </is>
+      </c>
+      <c r="O170" s="2" t="inlineStr">
+        <is>
+          <t>856612.8750186932</t>
+        </is>
+      </c>
+      <c r="P170" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q170" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R170" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S170" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T170" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U170" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V170" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W170" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X170" s="2" t="inlineStr">
+        <is>
+          <t>7973751.430000006</t>
+        </is>
+      </c>
+      <c r="Y170" s="2" t="inlineStr">
+        <is>
+          <t>118454044.3435051</t>
+        </is>
+      </c>
+      <c r="Z170" s="2" t="inlineStr">
+        <is>
+          <t>478698137.22633076</t>
+        </is>
+      </c>
+      <c r="AA170" s="2" t="inlineStr">
+        <is>
+          <t>1417715755.8518443</t>
+        </is>
+      </c>
+      <c r="AB170" s="2" t="inlineStr">
+        <is>
+          <t>7567</t>
+        </is>
+      </c>
+      <c r="AC170" s="2" t="inlineStr">
+        <is>
+          <t>66456</t>
+        </is>
+      </c>
+      <c r="AD170" s="2" t="inlineStr">
+        <is>
+          <t>264335</t>
+        </is>
+      </c>
+      <c r="AE170" s="2" t="inlineStr">
+        <is>
+          <t>738245</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-10-07
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE170"/>
+  <dimension ref="A1:AE171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27162,6 +27162,163 @@
         </is>
       </c>
     </row>
+    <row r="171">
+      <c r="A171" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B171" s="2" t="inlineStr">
+        <is>
+          <t>31678318044.26569</t>
+        </is>
+      </c>
+      <c r="C171" s="2" t="inlineStr">
+        <is>
+          <t>2350742620.4202957</t>
+        </is>
+      </c>
+      <c r="D171" s="2" t="inlineStr">
+        <is>
+          <t>80973</t>
+        </is>
+      </c>
+      <c r="E171" s="2" t="inlineStr">
+        <is>
+          <t>2349593642.3291564</t>
+        </is>
+      </c>
+      <c r="F171" s="2" t="inlineStr">
+        <is>
+          <t>24702812491.929996</t>
+        </is>
+      </c>
+      <c r="G171" s="2" t="inlineStr">
+        <is>
+          <t>396433</t>
+        </is>
+      </c>
+      <c r="H171" s="2" t="inlineStr">
+        <is>
+          <t>9082</t>
+        </is>
+      </c>
+      <c r="I171" s="2" t="inlineStr">
+        <is>
+          <t>76097</t>
+        </is>
+      </c>
+      <c r="J171" s="2" t="inlineStr">
+        <is>
+          <t>373054</t>
+        </is>
+      </c>
+      <c r="K171" s="2" t="inlineStr">
+        <is>
+          <t>1060823</t>
+        </is>
+      </c>
+      <c r="L171" s="2" t="inlineStr">
+        <is>
+          <t>1712.55500011139</t>
+        </is>
+      </c>
+      <c r="M171" s="2" t="inlineStr">
+        <is>
+          <t>49267.12766773896</t>
+        </is>
+      </c>
+      <c r="N171" s="2" t="inlineStr">
+        <is>
+          <t>257868.82667251446</t>
+        </is>
+      </c>
+      <c r="O171" s="2" t="inlineStr">
+        <is>
+          <t>853345.7283520049</t>
+        </is>
+      </c>
+      <c r="P171" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q171" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R171" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S171" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T171" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U171" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V171" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W171" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X171" s="2" t="inlineStr">
+        <is>
+          <t>6006925.301028567</t>
+        </is>
+      </c>
+      <c r="Y171" s="2" t="inlineStr">
+        <is>
+          <t>121589854.94350523</t>
+        </is>
+      </c>
+      <c r="Z171" s="2" t="inlineStr">
+        <is>
+          <t>492551551.51633084</t>
+        </is>
+      </c>
+      <c r="AA171" s="2" t="inlineStr">
+        <is>
+          <t>1426964589.8618443</t>
+        </is>
+      </c>
+      <c r="AB171" s="2" t="inlineStr">
+        <is>
+          <t>6261</t>
+        </is>
+      </c>
+      <c r="AC171" s="2" t="inlineStr">
+        <is>
+          <t>67467</t>
+        </is>
+      </c>
+      <c r="AD171" s="2" t="inlineStr">
+        <is>
+          <t>265306</t>
+        </is>
+      </c>
+      <c r="AE171" s="2" t="inlineStr">
+        <is>
+          <t>739248</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-10-08
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE171"/>
+  <dimension ref="A1:AE172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27319,6 +27319,163 @@
         </is>
       </c>
     </row>
+    <row r="172">
+      <c r="A172" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B172" s="2" t="inlineStr">
+        <is>
+          <t>31741039039.760506</t>
+        </is>
+      </c>
+      <c r="C172" s="2" t="inlineStr">
+        <is>
+          <t>2322580868.726453</t>
+        </is>
+      </c>
+      <c r="D172" s="2" t="inlineStr">
+        <is>
+          <t>81002</t>
+        </is>
+      </c>
+      <c r="E172" s="2" t="inlineStr">
+        <is>
+          <t>2322181664.323065</t>
+        </is>
+      </c>
+      <c r="F172" s="2" t="inlineStr">
+        <is>
+          <t>24775925354.41</t>
+        </is>
+      </c>
+      <c r="G172" s="2" t="inlineStr">
+        <is>
+          <t>397114</t>
+        </is>
+      </c>
+      <c r="H172" s="2" t="inlineStr">
+        <is>
+          <t>9803</t>
+        </is>
+      </c>
+      <c r="I172" s="2" t="inlineStr">
+        <is>
+          <t>77727</t>
+        </is>
+      </c>
+      <c r="J172" s="2" t="inlineStr">
+        <is>
+          <t>379838</t>
+        </is>
+      </c>
+      <c r="K172" s="2" t="inlineStr">
+        <is>
+          <t>1063232</t>
+        </is>
+      </c>
+      <c r="L172" s="2" t="inlineStr">
+        <is>
+          <t>3664.406889779585</t>
+        </is>
+      </c>
+      <c r="M172" s="2" t="inlineStr">
+        <is>
+          <t>48715.20600106293</t>
+        </is>
+      </c>
+      <c r="N172" s="2" t="inlineStr">
+        <is>
+          <t>265672.3833392856</t>
+        </is>
+      </c>
+      <c r="O172" s="2" t="inlineStr">
+        <is>
+          <t>851387.740685195</t>
+        </is>
+      </c>
+      <c r="P172" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q172" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R172" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S172" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T172" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U172" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V172" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W172" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X172" s="2" t="inlineStr">
+        <is>
+          <t>8069315.1000000145</t>
+        </is>
+      </c>
+      <c r="Y172" s="2" t="inlineStr">
+        <is>
+          <t>118896503.06102864</t>
+        </is>
+      </c>
+      <c r="Z172" s="2" t="inlineStr">
+        <is>
+          <t>501319848.0773593</t>
+        </is>
+      </c>
+      <c r="AA172" s="2" t="inlineStr">
+        <is>
+          <t>1430057840.6128728</t>
+        </is>
+      </c>
+      <c r="AB172" s="2" t="inlineStr">
+        <is>
+          <t>8552</t>
+        </is>
+      </c>
+      <c r="AC172" s="2" t="inlineStr">
+        <is>
+          <t>65061</t>
+        </is>
+      </c>
+      <c r="AD172" s="2" t="inlineStr">
+        <is>
+          <t>266061</t>
+        </is>
+      </c>
+      <c r="AE172" s="2" t="inlineStr">
+        <is>
+          <t>738930</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-10-09
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE172"/>
+  <dimension ref="A1:AE173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27476,6 +27476,163 @@
         </is>
       </c>
     </row>
+    <row r="173">
+      <c r="A173" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B173" s="2" t="inlineStr">
+        <is>
+          <t>31860146089.64292</t>
+        </is>
+      </c>
+      <c r="C173" s="2" t="inlineStr">
+        <is>
+          <t>2321502807.8188863</t>
+        </is>
+      </c>
+      <c r="D173" s="2" t="inlineStr">
+        <is>
+          <t>81029</t>
+        </is>
+      </c>
+      <c r="E173" s="2" t="inlineStr">
+        <is>
+          <t>2321626907.2601867</t>
+        </is>
+      </c>
+      <c r="F173" s="2" t="inlineStr">
+        <is>
+          <t>24835673537.820007</t>
+        </is>
+      </c>
+      <c r="G173" s="2" t="inlineStr">
+        <is>
+          <t>397721</t>
+        </is>
+      </c>
+      <c r="H173" s="2" t="inlineStr">
+        <is>
+          <t>8504</t>
+        </is>
+      </c>
+      <c r="I173" s="2" t="inlineStr">
+        <is>
+          <t>73273</t>
+        </is>
+      </c>
+      <c r="J173" s="2" t="inlineStr">
+        <is>
+          <t>374657</t>
+        </is>
+      </c>
+      <c r="K173" s="2" t="inlineStr">
+        <is>
+          <t>1070033</t>
+        </is>
+      </c>
+      <c r="L173" s="2" t="inlineStr">
+        <is>
+          <t>4669.242025608426</t>
+        </is>
+      </c>
+      <c r="M173" s="2" t="inlineStr">
+        <is>
+          <t>62765.58884989373</t>
+        </is>
+      </c>
+      <c r="N173" s="2" t="inlineStr">
+        <is>
+          <t>274862.7001881049</t>
+        </is>
+      </c>
+      <c r="O173" s="2" t="inlineStr">
+        <is>
+          <t>863058.8225339832</t>
+        </is>
+      </c>
+      <c r="P173" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q173" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R173" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S173" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T173" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U173" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V173" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W173" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X173" s="2" t="inlineStr">
+        <is>
+          <t>7382441.2800000105</t>
+        </is>
+      </c>
+      <c r="Y173" s="2" t="inlineStr">
+        <is>
+          <t>111717585.28102857</t>
+        </is>
+      </c>
+      <c r="Z173" s="2" t="inlineStr">
+        <is>
+          <t>504175620.21717405</t>
+        </is>
+      </c>
+      <c r="AA173" s="2" t="inlineStr">
+        <is>
+          <t>1435577909.262873</t>
+        </is>
+      </c>
+      <c r="AB173" s="2" t="inlineStr">
+        <is>
+          <t>7915</t>
+        </is>
+      </c>
+      <c r="AC173" s="2" t="inlineStr">
+        <is>
+          <t>61716</t>
+        </is>
+      </c>
+      <c r="AD173" s="2" t="inlineStr">
+        <is>
+          <t>267584</t>
+        </is>
+      </c>
+      <c r="AE173" s="2" t="inlineStr">
+        <is>
+          <t>740714</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-10-10
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE173"/>
+  <dimension ref="A1:AE174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27633,6 +27633,163 @@
         </is>
       </c>
     </row>
+    <row r="174">
+      <c r="A174" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B174" s="2" t="inlineStr">
+        <is>
+          <t>31905083643.1668</t>
+        </is>
+      </c>
+      <c r="C174" s="2" t="inlineStr">
+        <is>
+          <t>2331743789.807942</t>
+        </is>
+      </c>
+      <c r="D174" s="2" t="inlineStr">
+        <is>
+          <t>81055</t>
+        </is>
+      </c>
+      <c r="E174" s="2" t="inlineStr">
+        <is>
+          <t>2330926068.642235</t>
+        </is>
+      </c>
+      <c r="F174" s="2" t="inlineStr">
+        <is>
+          <t>24908487903.060013</t>
+        </is>
+      </c>
+      <c r="G174" s="2" t="inlineStr">
+        <is>
+          <t>398487</t>
+        </is>
+      </c>
+      <c r="H174" s="2" t="inlineStr">
+        <is>
+          <t>7853</t>
+        </is>
+      </c>
+      <c r="I174" s="2" t="inlineStr">
+        <is>
+          <t>76608</t>
+        </is>
+      </c>
+      <c r="J174" s="2" t="inlineStr">
+        <is>
+          <t>373143</t>
+        </is>
+      </c>
+      <c r="K174" s="2" t="inlineStr">
+        <is>
+          <t>1080255</t>
+        </is>
+      </c>
+      <c r="L174" s="2" t="inlineStr">
+        <is>
+          <t>2683.482076257695</t>
+        </is>
+      </c>
+      <c r="M174" s="2" t="inlineStr">
+        <is>
+          <t>69740.21672824855</t>
+        </is>
+      </c>
+      <c r="N174" s="2" t="inlineStr">
+        <is>
+          <t>281150.8627330702</t>
+        </is>
+      </c>
+      <c r="O174" s="2" t="inlineStr">
+        <is>
+          <t>877938.4344124357</t>
+        </is>
+      </c>
+      <c r="P174" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q174" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R174" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S174" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T174" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U174" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V174" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W174" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X174" s="2" t="inlineStr">
+        <is>
+          <t>563649.6699999997</t>
+        </is>
+      </c>
+      <c r="Y174" s="2" t="inlineStr">
+        <is>
+          <t>109740147.9310285</t>
+        </is>
+      </c>
+      <c r="Z174" s="2" t="inlineStr">
+        <is>
+          <t>501522321.9229687</t>
+        </is>
+      </c>
+      <c r="AA174" s="2" t="inlineStr">
+        <is>
+          <t>1443577388.6328728</t>
+        </is>
+      </c>
+      <c r="AB174" s="2" t="inlineStr">
+        <is>
+          <t>240</t>
+        </is>
+      </c>
+      <c r="AC174" s="2" t="inlineStr">
+        <is>
+          <t>60617</t>
+        </is>
+      </c>
+      <c r="AD174" s="2" t="inlineStr">
+        <is>
+          <t>268864</t>
+        </is>
+      </c>
+      <c r="AE174" s="2" t="inlineStr">
+        <is>
+          <t>743525</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-10-11
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE174"/>
+  <dimension ref="A1:AE175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27790,6 +27790,163 @@
         </is>
       </c>
     </row>
+    <row r="175">
+      <c r="A175" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B175" s="2" t="inlineStr">
+        <is>
+          <t>31923316767.25173</t>
+        </is>
+      </c>
+      <c r="C175" s="2" t="inlineStr">
+        <is>
+          <t>2334895024.356342</t>
+        </is>
+      </c>
+      <c r="D175" s="2" t="inlineStr">
+        <is>
+          <t>81076</t>
+        </is>
+      </c>
+      <c r="E175" s="2" t="inlineStr">
+        <is>
+          <t>2333641527.375552</t>
+        </is>
+      </c>
+      <c r="F175" s="2" t="inlineStr">
+        <is>
+          <t>24921619483.770004</t>
+        </is>
+      </c>
+      <c r="G175" s="2" t="inlineStr">
+        <is>
+          <t>398495</t>
+        </is>
+      </c>
+      <c r="H175" s="2" t="inlineStr">
+        <is>
+          <t>4145</t>
+        </is>
+      </c>
+      <c r="I175" s="2" t="inlineStr">
+        <is>
+          <t>81077</t>
+        </is>
+      </c>
+      <c r="J175" s="2" t="inlineStr">
+        <is>
+          <t>366478</t>
+        </is>
+      </c>
+      <c r="K175" s="2" t="inlineStr">
+        <is>
+          <t>1082132</t>
+        </is>
+      </c>
+      <c r="L175" s="2" t="inlineStr">
+        <is>
+          <t>479.07957218816</t>
+        </is>
+      </c>
+      <c r="M175" s="2" t="inlineStr">
+        <is>
+          <t>74111.3378223275</t>
+        </is>
+      </c>
+      <c r="N175" s="2" t="inlineStr">
+        <is>
+          <t>274782.867493627</t>
+        </is>
+      </c>
+      <c r="O175" s="2" t="inlineStr">
+        <is>
+          <t>883536.6631732429</t>
+        </is>
+      </c>
+      <c r="P175" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q175" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R175" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S175" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T175" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U175" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V175" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W175" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X175" s="2" t="inlineStr">
+        <is>
+          <t>5588790.350000004</t>
+        </is>
+      </c>
+      <c r="Y175" s="2" t="inlineStr">
+        <is>
+          <t>108353243.75102855</t>
+        </is>
+      </c>
+      <c r="Z175" s="2" t="inlineStr">
+        <is>
+          <t>493059512.4329688</t>
+        </is>
+      </c>
+      <c r="AA175" s="2" t="inlineStr">
+        <is>
+          <t>1446827430.2228727</t>
+        </is>
+      </c>
+      <c r="AB175" s="2" t="inlineStr">
+        <is>
+          <t>6979</t>
+        </is>
+      </c>
+      <c r="AC175" s="2" t="inlineStr">
+        <is>
+          <t>60964</t>
+        </is>
+      </c>
+      <c r="AD175" s="2" t="inlineStr">
+        <is>
+          <t>268487</t>
+        </is>
+      </c>
+      <c r="AE175" s="2" t="inlineStr">
+        <is>
+          <t>745920</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-10-12
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE175"/>
+  <dimension ref="A1:AE176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27947,6 +27947,163 @@
         </is>
       </c>
     </row>
+    <row r="176">
+      <c r="A176" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B176" s="2" t="inlineStr">
+        <is>
+          <t>31940121840.445717</t>
+        </is>
+      </c>
+      <c r="C176" s="2" t="inlineStr">
+        <is>
+          <t>2338795028.0469937</t>
+        </is>
+      </c>
+      <c r="D176" s="2" t="inlineStr">
+        <is>
+          <t>81108</t>
+        </is>
+      </c>
+      <c r="E176" s="2" t="inlineStr">
+        <is>
+          <t>2332980368.9728317</t>
+        </is>
+      </c>
+      <c r="F176" s="2" t="inlineStr">
+        <is>
+          <t>24919217059.029995</t>
+        </is>
+      </c>
+      <c r="G176" s="2" t="inlineStr">
+        <is>
+          <t>398468</t>
+        </is>
+      </c>
+      <c r="H176" s="2" t="inlineStr">
+        <is>
+          <t>3731</t>
+        </is>
+      </c>
+      <c r="I176" s="2" t="inlineStr">
+        <is>
+          <t>78205</t>
+        </is>
+      </c>
+      <c r="J176" s="2" t="inlineStr">
+        <is>
+          <t>362557</t>
+        </is>
+      </c>
+      <c r="K176" s="2" t="inlineStr">
+        <is>
+          <t>1071491</t>
+        </is>
+      </c>
+      <c r="L176" s="2" t="inlineStr">
+        <is>
+          <t>973.911597864984</t>
+        </is>
+      </c>
+      <c r="M176" s="2" t="inlineStr">
+        <is>
+          <t>76718.36474832031</t>
+        </is>
+      </c>
+      <c r="N176" s="2" t="inlineStr">
+        <is>
+          <t>265016.54308600293</t>
+        </is>
+      </c>
+      <c r="O176" s="2" t="inlineStr">
+        <is>
+          <t>879248.2214324577</t>
+        </is>
+      </c>
+      <c r="P176" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q176" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R176" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S176" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T176" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U176" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V176" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W176" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X176" s="2" t="inlineStr">
+        <is>
+          <t>5889411.570000003</t>
+        </is>
+      </c>
+      <c r="Y176" s="2" t="inlineStr">
+        <is>
+          <t>108915028.76102856</t>
+        </is>
+      </c>
+      <c r="Z176" s="2" t="inlineStr">
+        <is>
+          <t>478635320.98296887</t>
+        </is>
+      </c>
+      <c r="AA176" s="2" t="inlineStr">
+        <is>
+          <t>1441787734.012873</t>
+        </is>
+      </c>
+      <c r="AB176" s="2" t="inlineStr">
+        <is>
+          <t>6762</t>
+        </is>
+      </c>
+      <c r="AC176" s="2" t="inlineStr">
+        <is>
+          <t>60902</t>
+        </is>
+      </c>
+      <c r="AD176" s="2" t="inlineStr">
+        <is>
+          <t>267031</t>
+        </is>
+      </c>
+      <c r="AE176" s="2" t="inlineStr">
+        <is>
+          <t>746286</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-10-13
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE176"/>
+  <dimension ref="A1:AE177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28104,6 +28104,163 @@
         </is>
       </c>
     </row>
+    <row r="177">
+      <c r="A177" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B177" s="2" t="inlineStr">
+        <is>
+          <t>31928785412.948154</t>
+        </is>
+      </c>
+      <c r="C177" s="2" t="inlineStr">
+        <is>
+          <t>2328288430.051532</t>
+        </is>
+      </c>
+      <c r="D177" s="2" t="inlineStr">
+        <is>
+          <t>81128</t>
+        </is>
+      </c>
+      <c r="E177" s="2" t="inlineStr">
+        <is>
+          <t>2325719936.3749557</t>
+        </is>
+      </c>
+      <c r="F177" s="2" t="inlineStr">
+        <is>
+          <t>24913543189.18</t>
+        </is>
+      </c>
+      <c r="G177" s="2" t="inlineStr">
+        <is>
+          <t>398408</t>
+        </is>
+      </c>
+      <c r="H177" s="2" t="inlineStr">
+        <is>
+          <t>4137</t>
+        </is>
+      </c>
+      <c r="I177" s="2" t="inlineStr">
+        <is>
+          <t>65532</t>
+        </is>
+      </c>
+      <c r="J177" s="2" t="inlineStr">
+        <is>
+          <t>363551</t>
+        </is>
+      </c>
+      <c r="K177" s="2" t="inlineStr">
+        <is>
+          <t>1064430</t>
+        </is>
+      </c>
+      <c r="L177" s="2" t="inlineStr">
+        <is>
+          <t>750.593547507864</t>
+        </is>
+      </c>
+      <c r="M177" s="2" t="inlineStr">
+        <is>
+          <t>83533.6057445211</t>
+        </is>
+      </c>
+      <c r="N177" s="2" t="inlineStr">
+        <is>
+          <t>273937.3674154824</t>
+        </is>
+      </c>
+      <c r="O177" s="2" t="inlineStr">
+        <is>
+          <t>876140.0324284091</t>
+        </is>
+      </c>
+      <c r="P177" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q177" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R177" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S177" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T177" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U177" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V177" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W177" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X177" s="2" t="inlineStr">
+        <is>
+          <t>6573053.909999994</t>
+        </is>
+      </c>
+      <c r="Y177" s="2" t="inlineStr">
+        <is>
+          <t>100077792.30102856</t>
+        </is>
+      </c>
+      <c r="Z177" s="2" t="inlineStr">
+        <is>
+          <t>478948964.17296886</t>
+        </is>
+      </c>
+      <c r="AA177" s="2" t="inlineStr">
+        <is>
+          <t>1436994736.252873</t>
+        </is>
+      </c>
+      <c r="AB177" s="2" t="inlineStr">
+        <is>
+          <t>7299</t>
+        </is>
+      </c>
+      <c r="AC177" s="2" t="inlineStr">
+        <is>
+          <t>60291</t>
+        </is>
+      </c>
+      <c r="AD177" s="2" t="inlineStr">
+        <is>
+          <t>267029</t>
+        </is>
+      </c>
+      <c r="AE177" s="2" t="inlineStr">
+        <is>
+          <t>747034</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-10-14
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE177"/>
+  <dimension ref="A1:AE178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28261,6 +28261,163 @@
         </is>
       </c>
     </row>
+    <row r="178">
+      <c r="A178" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B178" s="2" t="inlineStr">
+        <is>
+          <t>32083629748.87063</t>
+        </is>
+      </c>
+      <c r="C178" s="2" t="inlineStr">
+        <is>
+          <t>2335131039.4746113</t>
+        </is>
+      </c>
+      <c r="D178" s="2" t="inlineStr">
+        <is>
+          <t>81165</t>
+        </is>
+      </c>
+      <c r="E178" s="2" t="inlineStr">
+        <is>
+          <t>2334364938.3918734</t>
+        </is>
+      </c>
+      <c r="F178" s="2" t="inlineStr">
+        <is>
+          <t>25018933585.579998</t>
+        </is>
+      </c>
+      <c r="G178" s="2" t="inlineStr">
+        <is>
+          <t>400054</t>
+        </is>
+      </c>
+      <c r="H178" s="2" t="inlineStr">
+        <is>
+          <t>12855</t>
+        </is>
+      </c>
+      <c r="I178" s="2" t="inlineStr">
+        <is>
+          <t>59162</t>
+        </is>
+      </c>
+      <c r="J178" s="2" t="inlineStr">
+        <is>
+          <t>362799</t>
+        </is>
+      </c>
+      <c r="K178" s="2" t="inlineStr">
+        <is>
+          <t>1059903</t>
+        </is>
+      </c>
+      <c r="L178" s="2" t="inlineStr">
+        <is>
+          <t>7105.081464531358</t>
+        </is>
+      </c>
+      <c r="M178" s="2" t="inlineStr">
+        <is>
+          <t>96437.9611307337</t>
+        </is>
+      </c>
+      <c r="N178" s="2" t="inlineStr">
+        <is>
+          <t>293989.811801806</t>
+        </is>
+      </c>
+      <c r="O178" s="2" t="inlineStr">
+        <is>
+          <t>888920.0301479176</t>
+        </is>
+      </c>
+      <c r="P178" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q178" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R178" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S178" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T178" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U178" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V178" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W178" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X178" s="2" t="inlineStr">
+        <is>
+          <t>786950.58</t>
+        </is>
+      </c>
+      <c r="Y178" s="2" t="inlineStr">
+        <is>
+          <t>96018721.29102843</t>
+        </is>
+      </c>
+      <c r="Z178" s="2" t="inlineStr">
+        <is>
+          <t>489932058.96296877</t>
+        </is>
+      </c>
+      <c r="AA178" s="2" t="inlineStr">
+        <is>
+          <t>1438402017.9728727</t>
+        </is>
+      </c>
+      <c r="AB178" s="2" t="inlineStr">
+        <is>
+          <t>233</t>
+        </is>
+      </c>
+      <c r="AC178" s="2" t="inlineStr">
+        <is>
+          <t>59828</t>
+        </is>
+      </c>
+      <c r="AD178" s="2" t="inlineStr">
+        <is>
+          <t>267682</t>
+        </is>
+      </c>
+      <c r="AE178" s="2" t="inlineStr">
+        <is>
+          <t>745869</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-10-15
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE178"/>
+  <dimension ref="A1:AE179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28418,6 +28418,163 @@
         </is>
       </c>
     </row>
+    <row r="179">
+      <c r="A179" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B179" s="2" t="inlineStr">
+        <is>
+          <t>32145989021.82426</t>
+        </is>
+      </c>
+      <c r="C179" s="2" t="inlineStr">
+        <is>
+          <t>2320737789.8177</t>
+        </is>
+      </c>
+      <c r="D179" s="2" t="inlineStr">
+        <is>
+          <t>81187</t>
+        </is>
+      </c>
+      <c r="E179" s="2" t="inlineStr">
+        <is>
+          <t>2320152508.3559875</t>
+        </is>
+      </c>
+      <c r="F179" s="2" t="inlineStr">
+        <is>
+          <t>25098839238.58999</t>
+        </is>
+      </c>
+      <c r="G179" s="2" t="inlineStr">
+        <is>
+          <t>400888</t>
+        </is>
+      </c>
+      <c r="H179" s="2" t="inlineStr">
+        <is>
+          <t>9733</t>
+        </is>
+      </c>
+      <c r="I179" s="2" t="inlineStr">
+        <is>
+          <t>63144</t>
+        </is>
+      </c>
+      <c r="J179" s="2" t="inlineStr">
+        <is>
+          <t>362890</t>
+        </is>
+      </c>
+      <c r="K179" s="2" t="inlineStr">
+        <is>
+          <t>1066120</t>
+        </is>
+      </c>
+      <c r="L179" s="2" t="inlineStr">
+        <is>
+          <t>3854.009705604072</t>
+        </is>
+      </c>
+      <c r="M179" s="2" t="inlineStr">
+        <is>
+          <t>108952.43084057569</t>
+        </is>
+      </c>
+      <c r="N179" s="2" t="inlineStr">
+        <is>
+          <t>304761.3945116391</t>
+        </is>
+      </c>
+      <c r="O179" s="2" t="inlineStr">
+        <is>
+          <t>897860.5255243215</t>
+        </is>
+      </c>
+      <c r="P179" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q179" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R179" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S179" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T179" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U179" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V179" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W179" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X179" s="2" t="inlineStr">
+        <is>
+          <t>1323110.9500000004</t>
+        </is>
+      </c>
+      <c r="Y179" s="2" t="inlineStr">
+        <is>
+          <t>101984545.06999993</t>
+        </is>
+      </c>
+      <c r="Z179" s="2" t="inlineStr">
+        <is>
+          <t>495448937.60296875</t>
+        </is>
+      </c>
+      <c r="AA179" s="2" t="inlineStr">
+        <is>
+          <t>1446797330.8228726</t>
+        </is>
+      </c>
+      <c r="AB179" s="2" t="inlineStr">
+        <is>
+          <t>317</t>
+        </is>
+      </c>
+      <c r="AC179" s="2" t="inlineStr">
+        <is>
+          <t>61732</t>
+        </is>
+      </c>
+      <c r="AD179" s="2" t="inlineStr">
+        <is>
+          <t>269080</t>
+        </is>
+      </c>
+      <c r="AE179" s="2" t="inlineStr">
+        <is>
+          <t>746960</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-10-16
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE179"/>
+  <dimension ref="A1:AE180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28575,6 +28575,163 @@
         </is>
       </c>
     </row>
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B180" s="2" t="inlineStr">
+        <is>
+          <t>32261038478.38122</t>
+        </is>
+      </c>
+      <c r="C180" s="2" t="inlineStr">
+        <is>
+          <t>2341421930.7103643</t>
+        </is>
+      </c>
+      <c r="D180" s="2" t="inlineStr">
+        <is>
+          <t>81215</t>
+        </is>
+      </c>
+      <c r="E180" s="2" t="inlineStr">
+        <is>
+          <t>2341015718.661583</t>
+        </is>
+      </c>
+      <c r="F180" s="2" t="inlineStr">
+        <is>
+          <t>25175792579.910004</t>
+        </is>
+      </c>
+      <c r="G180" s="2" t="inlineStr">
+        <is>
+          <t>401707</t>
+        </is>
+      </c>
+      <c r="H180" s="2" t="inlineStr">
+        <is>
+          <t>9159</t>
+        </is>
+      </c>
+      <c r="I180" s="2" t="inlineStr">
+        <is>
+          <t>65893</t>
+        </is>
+      </c>
+      <c r="J180" s="2" t="inlineStr">
+        <is>
+          <t>361908</t>
+        </is>
+      </c>
+      <c r="K180" s="2" t="inlineStr">
+        <is>
+          <t>1074556</t>
+        </is>
+      </c>
+      <c r="L180" s="2" t="inlineStr">
+        <is>
+          <t>4212.615195588876</t>
+        </is>
+      </c>
+      <c r="M180" s="2" t="inlineStr">
+        <is>
+          <t>105299.90688447017</t>
+        </is>
+      </c>
+      <c r="N180" s="2" t="inlineStr">
+        <is>
+          <t>307911.98440419976</t>
+        </is>
+      </c>
+      <c r="O180" s="2" t="inlineStr">
+        <is>
+          <t>901577.9447502835</t>
+        </is>
+      </c>
+      <c r="P180" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q180" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R180" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S180" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T180" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U180" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V180" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W180" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X180" s="2" t="inlineStr">
+        <is>
+          <t>1449705.0599999996</t>
+        </is>
+      </c>
+      <c r="Y180" s="2" t="inlineStr">
+        <is>
+          <t>106085497.38999987</t>
+        </is>
+      </c>
+      <c r="Z180" s="2" t="inlineStr">
+        <is>
+          <t>498937876.48296875</t>
+        </is>
+      </c>
+      <c r="AA180" s="2" t="inlineStr">
+        <is>
+          <t>1455924892.4928727</t>
+        </is>
+      </c>
+      <c r="AB180" s="2" t="inlineStr">
+        <is>
+          <t>392</t>
+        </is>
+      </c>
+      <c r="AC180" s="2" t="inlineStr">
+        <is>
+          <t>63178</t>
+        </is>
+      </c>
+      <c r="AD180" s="2" t="inlineStr">
+        <is>
+          <t>270403</t>
+        </is>
+      </c>
+      <c r="AE180" s="2" t="inlineStr">
+        <is>
+          <t>749015</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-10-17
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE180"/>
+  <dimension ref="A1:AE181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28732,6 +28732,163 @@
         </is>
       </c>
     </row>
+    <row r="181">
+      <c r="A181" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B181" s="2" t="inlineStr">
+        <is>
+          <t>32362253405.854214</t>
+        </is>
+      </c>
+      <c r="C181" s="2" t="inlineStr">
+        <is>
+          <t>2337367914.775661</t>
+        </is>
+      </c>
+      <c r="D181" s="2" t="inlineStr">
+        <is>
+          <t>81238</t>
+        </is>
+      </c>
+      <c r="E181" s="2" t="inlineStr">
+        <is>
+          <t>2336782035.668261</t>
+        </is>
+      </c>
+      <c r="F181" s="2" t="inlineStr">
+        <is>
+          <t>25263133735.600002</t>
+        </is>
+      </c>
+      <c r="G181" s="2" t="inlineStr">
+        <is>
+          <t>402673</t>
+        </is>
+      </c>
+      <c r="H181" s="2" t="inlineStr">
+        <is>
+          <t>9197</t>
+        </is>
+      </c>
+      <c r="I181" s="2" t="inlineStr">
+        <is>
+          <t>72734</t>
+        </is>
+      </c>
+      <c r="J181" s="2" t="inlineStr">
+        <is>
+          <t>363734</t>
+        </is>
+      </c>
+      <c r="K181" s="2" t="inlineStr">
+        <is>
+          <t>1086632</t>
+        </is>
+      </c>
+      <c r="L181" s="2" t="inlineStr">
+        <is>
+          <t>3249.258135171432</t>
+        </is>
+      </c>
+      <c r="M181" s="2" t="inlineStr">
+        <is>
+          <t>107297.55073379705</t>
+        </is>
+      </c>
+      <c r="N181" s="2" t="inlineStr">
+        <is>
+          <t>316608.76546518103</t>
+        </is>
+      </c>
+      <c r="O181" s="2" t="inlineStr">
+        <is>
+          <t>918313.1018113855</t>
+        </is>
+      </c>
+      <c r="P181" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q181" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R181" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S181" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T181" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U181" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V181" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W181" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X181" s="2" t="inlineStr">
+        <is>
+          <t>719553.1299999997</t>
+        </is>
+      </c>
+      <c r="Y181" s="2" t="inlineStr">
+        <is>
+          <t>116617765.10999992</t>
+        </is>
+      </c>
+      <c r="Z181" s="2" t="inlineStr">
+        <is>
+          <t>503498306.7529688</t>
+        </is>
+      </c>
+      <c r="AA181" s="2" t="inlineStr">
+        <is>
+          <t>1472696307.8728726</t>
+        </is>
+      </c>
+      <c r="AB181" s="2" t="inlineStr">
+        <is>
+          <t>194</t>
+        </is>
+      </c>
+      <c r="AC181" s="2" t="inlineStr">
+        <is>
+          <t>63877</t>
+        </is>
+      </c>
+      <c r="AD181" s="2" t="inlineStr">
+        <is>
+          <t>272104</t>
+        </is>
+      </c>
+      <c r="AE181" s="2" t="inlineStr">
+        <is>
+          <t>751416</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-10-18
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE181"/>
+  <dimension ref="A1:AE182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28889,6 +28889,163 @@
         </is>
       </c>
     </row>
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B182" s="2" t="inlineStr">
+        <is>
+          <t>32376814099.744553</t>
+        </is>
+      </c>
+      <c r="C182" s="2" t="inlineStr">
+        <is>
+          <t>2337090609.9712543</t>
+        </is>
+      </c>
+      <c r="D182" s="2" t="inlineStr">
+        <is>
+          <t>81259</t>
+        </is>
+      </c>
+      <c r="E182" s="2" t="inlineStr">
+        <is>
+          <t>2335475163.7429132</t>
+        </is>
+      </c>
+      <c r="F182" s="2" t="inlineStr">
+        <is>
+          <t>25276745218.480015</t>
+        </is>
+      </c>
+      <c r="G182" s="2" t="inlineStr">
+        <is>
+          <t>402712</t>
+        </is>
+      </c>
+      <c r="H182" s="2" t="inlineStr">
+        <is>
+          <t>3890</t>
+        </is>
+      </c>
+      <c r="I182" s="2" t="inlineStr">
+        <is>
+          <t>78472</t>
+        </is>
+      </c>
+      <c r="J182" s="2" t="inlineStr">
+        <is>
+          <t>360751</t>
+        </is>
+      </c>
+      <c r="K182" s="2" t="inlineStr">
+        <is>
+          <t>1089632</t>
+        </is>
+      </c>
+      <c r="L182" s="2" t="inlineStr">
+        <is>
+          <t>543.186623144736</t>
+        </is>
+      </c>
+      <c r="M182" s="2" t="inlineStr">
+        <is>
+          <t>108088.45612270417</t>
+        </is>
+      </c>
+      <c r="N182" s="2" t="inlineStr">
+        <is>
+          <t>313428.64628141903</t>
+        </is>
+      </c>
+      <c r="O182" s="2" t="inlineStr">
+        <is>
+          <t>924523.3212944232</t>
+        </is>
+      </c>
+      <c r="P182" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q182" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R182" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S182" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T182" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U182" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V182" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W182" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X182" s="2" t="inlineStr">
+        <is>
+          <t>870708.8599999996</t>
+        </is>
+      </c>
+      <c r="Y182" s="2" t="inlineStr">
+        <is>
+          <t>118181345.72999983</t>
+        </is>
+      </c>
+      <c r="Z182" s="2" t="inlineStr">
+        <is>
+          <t>490327318.2329686</t>
+        </is>
+      </c>
+      <c r="AA182" s="2" t="inlineStr">
+        <is>
+          <t>1479285508.9228725</t>
+        </is>
+      </c>
+      <c r="AB182" s="2" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="AC182" s="2" t="inlineStr">
+        <is>
+          <t>64913</t>
+        </is>
+      </c>
+      <c r="AD182" s="2" t="inlineStr">
+        <is>
+          <t>271491</t>
+        </is>
+      </c>
+      <c r="AE182" s="2" t="inlineStr">
+        <is>
+          <t>756345</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-10-19
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE182"/>
+  <dimension ref="A1:AE183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29046,6 +29046,163 @@
         </is>
       </c>
     </row>
+    <row r="183">
+      <c r="A183" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B183" s="2" t="inlineStr">
+        <is>
+          <t>32400202348.669453</t>
+        </is>
+      </c>
+      <c r="C183" s="2" t="inlineStr">
+        <is>
+          <t>2343308130.4520116</t>
+        </is>
+      </c>
+      <c r="D183" s="2" t="inlineStr">
+        <is>
+          <t>81276</t>
+        </is>
+      </c>
+      <c r="E183" s="2" t="inlineStr">
+        <is>
+          <t>2339468766.4717116</t>
+        </is>
+      </c>
+      <c r="F183" s="2" t="inlineStr">
+        <is>
+          <t>25272847403.31001</t>
+        </is>
+      </c>
+      <c r="G183" s="2" t="inlineStr">
+        <is>
+          <t>402605</t>
+        </is>
+      </c>
+      <c r="H183" s="2" t="inlineStr">
+        <is>
+          <t>3664</t>
+        </is>
+      </c>
+      <c r="I183" s="2" t="inlineStr">
+        <is>
+          <t>77395</t>
+        </is>
+      </c>
+      <c r="J183" s="2" t="inlineStr">
+        <is>
+          <t>355301</t>
+        </is>
+      </c>
+      <c r="K183" s="2" t="inlineStr">
+        <is>
+          <t>1075205</t>
+        </is>
+      </c>
+      <c r="L183" s="2" t="inlineStr">
+        <is>
+          <t>703.6274022484</t>
+        </is>
+      </c>
+      <c r="M183" s="2" t="inlineStr">
+        <is>
+          <t>108115.91317219025</t>
+        </is>
+      </c>
+      <c r="N183" s="2" t="inlineStr">
+        <is>
+          <t>306017.02559003833</t>
+        </is>
+      </c>
+      <c r="O183" s="2" t="inlineStr">
+        <is>
+          <t>919503.7179364609</t>
+        </is>
+      </c>
+      <c r="P183" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q183" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R183" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S183" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T183" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U183" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V183" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W183" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X183" s="2" t="inlineStr">
+        <is>
+          <t>4893947.05999999</t>
+        </is>
+      </c>
+      <c r="Y183" s="2" t="inlineStr">
+        <is>
+          <t>119235743.18999983</t>
+        </is>
+      </c>
+      <c r="Z183" s="2" t="inlineStr">
+        <is>
+          <t>480767397.0029686</t>
+        </is>
+      </c>
+      <c r="AA183" s="2" t="inlineStr">
+        <is>
+          <t>1470821217.4828727</t>
+        </is>
+      </c>
+      <c r="AB183" s="2" t="inlineStr">
+        <is>
+          <t>5404</t>
+        </is>
+      </c>
+      <c r="AC183" s="2" t="inlineStr">
+        <is>
+          <t>65999</t>
+        </is>
+      </c>
+      <c r="AD183" s="2" t="inlineStr">
+        <is>
+          <t>270166</t>
+        </is>
+      </c>
+      <c r="AE183" s="2" t="inlineStr">
+        <is>
+          <t>756882</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-10-20
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE183"/>
+  <dimension ref="A1:AE184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29203,6 +29203,163 @@
         </is>
       </c>
     </row>
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B184" s="2" t="inlineStr">
+        <is>
+          <t>32509290094.093678</t>
+        </is>
+      </c>
+      <c r="C184" s="2" t="inlineStr">
+        <is>
+          <t>2338599568.2625036</t>
+        </is>
+      </c>
+      <c r="D184" s="2" t="inlineStr">
+        <is>
+          <t>81293</t>
+        </is>
+      </c>
+      <c r="E184" s="2" t="inlineStr">
+        <is>
+          <t>2338316555.8798246</t>
+        </is>
+      </c>
+      <c r="F184" s="2" t="inlineStr">
+        <is>
+          <t>25259647212.229992</t>
+        </is>
+      </c>
+      <c r="G184" s="2" t="inlineStr">
+        <is>
+          <t>402801</t>
+        </is>
+      </c>
+      <c r="H184" s="2" t="inlineStr">
+        <is>
+          <t>9889</t>
+        </is>
+      </c>
+      <c r="I184" s="2" t="inlineStr">
+        <is>
+          <t>77941</t>
+        </is>
+      </c>
+      <c r="J184" s="2" t="inlineStr">
+        <is>
+          <t>360252</t>
+        </is>
+      </c>
+      <c r="K184" s="2" t="inlineStr">
+        <is>
+          <t>1067847</t>
+        </is>
+      </c>
+      <c r="L184" s="2" t="inlineStr">
+        <is>
+          <t>4364.40804491796</t>
+        </is>
+      </c>
+      <c r="M184" s="2" t="inlineStr">
+        <is>
+          <t>108567.43035491685</t>
+        </is>
+      </c>
+      <c r="N184" s="2" t="inlineStr">
+        <is>
+          <t>315813.7141022063</t>
+        </is>
+      </c>
+      <c r="O184" s="2" t="inlineStr">
+        <is>
+          <t>898385.1854483599</t>
+        </is>
+      </c>
+      <c r="P184" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q184" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R184" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S184" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T184" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U184" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V184" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W184" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X184" s="2" t="inlineStr">
+        <is>
+          <t>1121657.55</t>
+        </is>
+      </c>
+      <c r="Y184" s="2" t="inlineStr">
+        <is>
+          <t>123199937.53999981</t>
+        </is>
+      </c>
+      <c r="Z184" s="2" t="inlineStr">
+        <is>
+          <t>487591081.2329686</t>
+        </is>
+      </c>
+      <c r="AA184" s="2" t="inlineStr">
+        <is>
+          <t>1461857277.8728726</t>
+        </is>
+      </c>
+      <c r="AB184" s="2" t="inlineStr">
+        <is>
+          <t>214</t>
+        </is>
+      </c>
+      <c r="AC184" s="2" t="inlineStr">
+        <is>
+          <t>65131</t>
+        </is>
+      </c>
+      <c r="AD184" s="2" t="inlineStr">
+        <is>
+          <t>270701</t>
+        </is>
+      </c>
+      <c r="AE184" s="2" t="inlineStr">
+        <is>
+          <t>756890</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-10-21
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE184"/>
+  <dimension ref="A1:AE185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29360,6 +29360,163 @@
         </is>
       </c>
     </row>
+    <row r="185">
+      <c r="A185" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B185" s="2" t="inlineStr">
+        <is>
+          <t>32603686578.52945</t>
+        </is>
+      </c>
+      <c r="C185" s="2" t="inlineStr">
+        <is>
+          <t>2340709786.582466</t>
+        </is>
+      </c>
+      <c r="D185" s="2" t="inlineStr">
+        <is>
+          <t>81340</t>
+        </is>
+      </c>
+      <c r="E185" s="2" t="inlineStr">
+        <is>
+          <t>2340663568.8502483</t>
+        </is>
+      </c>
+      <c r="F185" s="2" t="inlineStr">
+        <is>
+          <t>25441104262.03</t>
+        </is>
+      </c>
+      <c r="G185" s="2" t="inlineStr">
+        <is>
+          <t>404903</t>
+        </is>
+      </c>
+      <c r="H185" s="2" t="inlineStr">
+        <is>
+          <t>8142</t>
+        </is>
+      </c>
+      <c r="I185" s="2" t="inlineStr">
+        <is>
+          <t>77512</t>
+        </is>
+      </c>
+      <c r="J185" s="2" t="inlineStr">
+        <is>
+          <t>370122</t>
+        </is>
+      </c>
+      <c r="K185" s="2" t="inlineStr">
+        <is>
+          <t>1072658</t>
+        </is>
+      </c>
+      <c r="L185" s="2" t="inlineStr">
+        <is>
+          <t>3723.817770997625</t>
+        </is>
+      </c>
+      <c r="M185" s="2" t="inlineStr">
+        <is>
+          <t>109545.76460208271</t>
+        </is>
+      </c>
+      <c r="N185" s="2" t="inlineStr">
+        <is>
+          <t>337038.9107357186</t>
+        </is>
+      </c>
+      <c r="O185" s="2" t="inlineStr">
+        <is>
+          <t>877348.4364148394</t>
+        </is>
+      </c>
+      <c r="P185" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q185" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R185" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S185" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T185" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U185" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V185" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W185" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X185" s="2" t="inlineStr">
+        <is>
+          <t>2013596.3199999994</t>
+        </is>
+      </c>
+      <c r="Y185" s="2" t="inlineStr">
+        <is>
+          <t>126958224.78999987</t>
+        </is>
+      </c>
+      <c r="Z185" s="2" t="inlineStr">
+        <is>
+          <t>501098229.7229686</t>
+        </is>
+      </c>
+      <c r="AA185" s="2" t="inlineStr">
+        <is>
+          <t>1470408909.2528725</t>
+        </is>
+      </c>
+      <c r="AB185" s="2" t="inlineStr">
+        <is>
+          <t>278</t>
+        </is>
+      </c>
+      <c r="AC185" s="2" t="inlineStr">
+        <is>
+          <t>66254</t>
+        </is>
+      </c>
+      <c r="AD185" s="2" t="inlineStr">
+        <is>
+          <t>271535</t>
+        </is>
+      </c>
+      <c r="AE185" s="2" t="inlineStr">
+        <is>
+          <t>758098</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-10-22
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE185"/>
+  <dimension ref="A1:AE186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29517,6 +29517,163 @@
         </is>
       </c>
     </row>
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B186" s="2" t="inlineStr">
+        <is>
+          <t>33284345772.68448</t>
+        </is>
+      </c>
+      <c r="C186" s="2" t="inlineStr">
+        <is>
+          <t>2330163755.7540336</t>
+        </is>
+      </c>
+      <c r="D186" s="2" t="inlineStr">
+        <is>
+          <t>81378</t>
+        </is>
+      </c>
+      <c r="E186" s="2" t="inlineStr">
+        <is>
+          <t>2326410405.4325557</t>
+        </is>
+      </c>
+      <c r="F186" s="2" t="inlineStr">
+        <is>
+          <t>25522155461.179993</t>
+        </is>
+      </c>
+      <c r="G186" s="2" t="inlineStr">
+        <is>
+          <t>405792</t>
+        </is>
+      </c>
+      <c r="H186" s="2" t="inlineStr">
+        <is>
+          <t>9054</t>
+        </is>
+      </c>
+      <c r="I186" s="2" t="inlineStr">
+        <is>
+          <t>78174</t>
+        </is>
+      </c>
+      <c r="J186" s="2" t="inlineStr">
+        <is>
+          <t>369466</t>
+        </is>
+      </c>
+      <c r="K186" s="2" t="inlineStr">
+        <is>
+          <t>1078232</t>
+        </is>
+      </c>
+      <c r="L186" s="2" t="inlineStr">
+        <is>
+          <t>3747.7780207988585</t>
+        </is>
+      </c>
+      <c r="M186" s="2" t="inlineStr">
+        <is>
+          <t>106243.80102789999</t>
+        </is>
+      </c>
+      <c r="N186" s="2" t="inlineStr">
+        <is>
+          <t>344811.44320473255</t>
+        </is>
+      </c>
+      <c r="O186" s="2" t="inlineStr">
+        <is>
+          <t>884924.4375504182</t>
+        </is>
+      </c>
+      <c r="P186" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q186" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R186" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S186" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T186" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U186" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V186" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W186" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X186" s="2" t="inlineStr">
+        <is>
+          <t>1374156.0499999998</t>
+        </is>
+      </c>
+      <c r="Y186" s="2" t="inlineStr">
+        <is>
+          <t>127555424.63493443</t>
+        </is>
+      </c>
+      <c r="Z186" s="2" t="inlineStr">
+        <is>
+          <t>511853126.5679032</t>
+        </is>
+      </c>
+      <c r="AA186" s="2" t="inlineStr">
+        <is>
+          <t>1466839090.9278069</t>
+        </is>
+      </c>
+      <c r="AB186" s="2" t="inlineStr">
+        <is>
+          <t>269</t>
+        </is>
+      </c>
+      <c r="AC186" s="2" t="inlineStr">
+        <is>
+          <t>66199</t>
+        </is>
+      </c>
+      <c r="AD186" s="2" t="inlineStr">
+        <is>
+          <t>273111</t>
+        </is>
+      </c>
+      <c r="AE186" s="2" t="inlineStr">
+        <is>
+          <t>758937</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-10-23
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE186"/>
+  <dimension ref="A1:AE187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29674,6 +29674,163 @@
         </is>
       </c>
     </row>
+    <row r="187">
+      <c r="A187" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B187" s="2" t="inlineStr">
+        <is>
+          <t>33361246648.0617</t>
+        </is>
+      </c>
+      <c r="C187" s="2" t="inlineStr">
+        <is>
+          <t>2333220490.365895</t>
+        </is>
+      </c>
+      <c r="D187" s="2" t="inlineStr">
+        <is>
+          <t>81412</t>
+        </is>
+      </c>
+      <c r="E187" s="2" t="inlineStr">
+        <is>
+          <t>2332034477.8039746</t>
+        </is>
+      </c>
+      <c r="F187" s="2" t="inlineStr">
+        <is>
+          <t>25538676890.010002</t>
+        </is>
+      </c>
+      <c r="G187" s="2" t="inlineStr">
+        <is>
+          <t>405984</t>
+        </is>
+      </c>
+      <c r="H187" s="2" t="inlineStr">
+        <is>
+          <t>8343</t>
+        </is>
+      </c>
+      <c r="I187" s="2" t="inlineStr">
+        <is>
+          <t>76582</t>
+        </is>
+      </c>
+      <c r="J187" s="2" t="inlineStr">
+        <is>
+          <t>367500</t>
+        </is>
+      </c>
+      <c r="K187" s="2" t="inlineStr">
+        <is>
+          <t>1084507</t>
+        </is>
+      </c>
+      <c r="L187" s="2" t="inlineStr">
+        <is>
+          <t>4216.152508435159</t>
+        </is>
+      </c>
+      <c r="M187" s="2" t="inlineStr">
+        <is>
+          <t>108546.05599569078</t>
+        </is>
+      </c>
+      <c r="N187" s="2" t="inlineStr">
+        <is>
+          <t>351212.1043984491</t>
+        </is>
+      </c>
+      <c r="O187" s="2" t="inlineStr">
+        <is>
+          <t>892409.2934108411</t>
+        </is>
+      </c>
+      <c r="P187" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q187" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R187" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S187" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T187" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U187" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V187" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W187" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X187" s="2" t="inlineStr">
+        <is>
+          <t>1974125.5999999987</t>
+        </is>
+      </c>
+      <c r="Y187" s="2" t="inlineStr">
+        <is>
+          <t>127114096.85755152</t>
+        </is>
+      </c>
+      <c r="Z187" s="2" t="inlineStr">
+        <is>
+          <t>512546516.16052026</t>
+        </is>
+      </c>
+      <c r="AA187" s="2" t="inlineStr">
+        <is>
+          <t>1471675269.4477098</t>
+        </is>
+      </c>
+      <c r="AB187" s="2" t="inlineStr">
+        <is>
+          <t>332</t>
+        </is>
+      </c>
+      <c r="AC187" s="2" t="inlineStr">
+        <is>
+          <t>64653</t>
+        </is>
+      </c>
+      <c r="AD187" s="2" t="inlineStr">
+        <is>
+          <t>274201</t>
+        </is>
+      </c>
+      <c r="AE187" s="2" t="inlineStr">
+        <is>
+          <t>759696</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-10-24
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE187"/>
+  <dimension ref="A1:AE188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29831,6 +29831,163 @@
         </is>
       </c>
     </row>
+    <row r="188">
+      <c r="A188" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B188" s="2" t="inlineStr">
+        <is>
+          <t>33424952189.370453</t>
+        </is>
+      </c>
+      <c r="C188" s="2" t="inlineStr">
+        <is>
+          <t>2325417766.8196177</t>
+        </is>
+      </c>
+      <c r="D188" s="2" t="inlineStr">
+        <is>
+          <t>81434</t>
+        </is>
+      </c>
+      <c r="E188" s="2" t="inlineStr">
+        <is>
+          <t>2324056306.2842226</t>
+        </is>
+      </c>
+      <c r="F188" s="2" t="inlineStr">
+        <is>
+          <t>25616211386.890003</t>
+        </is>
+      </c>
+      <c r="G188" s="2" t="inlineStr">
+        <is>
+          <t>406940</t>
+        </is>
+      </c>
+      <c r="H188" s="2" t="inlineStr">
+        <is>
+          <t>8010</t>
+        </is>
+      </c>
+      <c r="I188" s="2" t="inlineStr">
+        <is>
+          <t>78458</t>
+        </is>
+      </c>
+      <c r="J188" s="2" t="inlineStr">
+        <is>
+          <t>365121</t>
+        </is>
+      </c>
+      <c r="K188" s="2" t="inlineStr">
+        <is>
+          <t>1093375</t>
+        </is>
+      </c>
+      <c r="L188" s="2" t="inlineStr">
+        <is>
+          <t>2586.543792446753</t>
+        </is>
+      </c>
+      <c r="M188" s="2" t="inlineStr">
+        <is>
+          <t>104795.21918805531</t>
+        </is>
+      </c>
+      <c r="N188" s="2" t="inlineStr">
+        <is>
+          <t>356584.2016518108</t>
+        </is>
+      </c>
+      <c r="O188" s="2" t="inlineStr">
+        <is>
+          <t>904646.522997646</t>
+        </is>
+      </c>
+      <c r="P188" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q188" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R188" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S188" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T188" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U188" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V188" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W188" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X188" s="2" t="inlineStr">
+        <is>
+          <t>905314.02</t>
+        </is>
+      </c>
+      <c r="Y188" s="2" t="inlineStr">
+        <is>
+          <t>116773612.79755157</t>
+        </is>
+      </c>
+      <c r="Z188" s="2" t="inlineStr">
+        <is>
+          <t>508521553.1905202</t>
+        </is>
+      </c>
+      <c r="AA188" s="2" t="inlineStr">
+        <is>
+          <t>1478992912.59771</t>
+        </is>
+      </c>
+      <c r="AB188" s="2" t="inlineStr">
+        <is>
+          <t>215</t>
+        </is>
+      </c>
+      <c r="AC188" s="2" t="inlineStr">
+        <is>
+          <t>64576</t>
+        </is>
+      </c>
+      <c r="AD188" s="2" t="inlineStr">
+        <is>
+          <t>275717</t>
+        </is>
+      </c>
+      <c r="AE188" s="2" t="inlineStr">
+        <is>
+          <t>763593</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-10-25
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE188"/>
+  <dimension ref="A1:AE189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29988,6 +29988,163 @@
         </is>
       </c>
     </row>
+    <row r="189">
+      <c r="A189" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B189" s="2" t="inlineStr">
+        <is>
+          <t>33439150959.56402</t>
+        </is>
+      </c>
+      <c r="C189" s="2" t="inlineStr">
+        <is>
+          <t>2320275593.390695</t>
+        </is>
+      </c>
+      <c r="D189" s="2" t="inlineStr">
+        <is>
+          <t>81447</t>
+        </is>
+      </c>
+      <c r="E189" s="2" t="inlineStr">
+        <is>
+          <t>2320092414.857347</t>
+        </is>
+      </c>
+      <c r="F189" s="2" t="inlineStr">
+        <is>
+          <t>25637696068.5</t>
+        </is>
+      </c>
+      <c r="G189" s="2" t="inlineStr">
+        <is>
+          <t>407011</t>
+        </is>
+      </c>
+      <c r="H189" s="2" t="inlineStr">
+        <is>
+          <t>4151</t>
+        </is>
+      </c>
+      <c r="I189" s="2" t="inlineStr">
+        <is>
+          <t>83203</t>
+        </is>
+      </c>
+      <c r="J189" s="2" t="inlineStr">
+        <is>
+          <t>357843</t>
+        </is>
+      </c>
+      <c r="K189" s="2" t="inlineStr">
+        <is>
+          <t>1094127</t>
+        </is>
+      </c>
+      <c r="L189" s="2" t="inlineStr">
+        <is>
+          <t>615.7709033209185</t>
+        </is>
+      </c>
+      <c r="M189" s="2" t="inlineStr">
+        <is>
+          <t>104751.38549850532</t>
+        </is>
+      </c>
+      <c r="N189" s="2" t="inlineStr">
+        <is>
+          <t>355579.9534451396</t>
+        </is>
+      </c>
+      <c r="O189" s="2" t="inlineStr">
+        <is>
+          <t>910569.879791133</t>
+        </is>
+      </c>
+      <c r="P189" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q189" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R189" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S189" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T189" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U189" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V189" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W189" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X189" s="2" t="inlineStr">
+        <is>
+          <t>468038.46000000014</t>
+        </is>
+      </c>
+      <c r="Y189" s="2" t="inlineStr">
+        <is>
+          <t>115504791.70325212</t>
+        </is>
+      </c>
+      <c r="Z189" s="2" t="inlineStr">
+        <is>
+          <t>496432664.6562209</t>
+        </is>
+      </c>
+      <c r="AA189" s="2" t="inlineStr">
+        <is>
+          <t>1480739788.2034104</t>
+        </is>
+      </c>
+      <c r="AB189" s="2" t="inlineStr">
+        <is>
+          <t>118</t>
+        </is>
+      </c>
+      <c r="AC189" s="2" t="inlineStr">
+        <is>
+          <t>64159</t>
+        </is>
+      </c>
+      <c r="AD189" s="2" t="inlineStr">
+        <is>
+          <t>275281</t>
+        </is>
+      </c>
+      <c r="AE189" s="2" t="inlineStr">
+        <is>
+          <t>766181</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-10-26
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE189"/>
+  <dimension ref="A1:AE190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30145,6 +30145,163 @@
         </is>
       </c>
     </row>
+    <row r="190">
+      <c r="A190" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B190" s="2" t="inlineStr">
+        <is>
+          <t>33439385822.04612</t>
+        </is>
+      </c>
+      <c r="C190" s="2" t="inlineStr">
+        <is>
+          <t>2322078948.4678903</t>
+        </is>
+      </c>
+      <c r="D190" s="2" t="inlineStr">
+        <is>
+          <t>81470</t>
+        </is>
+      </c>
+      <c r="E190" s="2" t="inlineStr">
+        <is>
+          <t>2319340659.5180025</t>
+        </is>
+      </c>
+      <c r="F190" s="2" t="inlineStr">
+        <is>
+          <t>25633354348.550003</t>
+        </is>
+      </c>
+      <c r="G190" s="2" t="inlineStr">
+        <is>
+          <t>406971</t>
+        </is>
+      </c>
+      <c r="H190" s="2" t="inlineStr">
+        <is>
+          <t>3836</t>
+        </is>
+      </c>
+      <c r="I190" s="2" t="inlineStr">
+        <is>
+          <t>78969</t>
+        </is>
+      </c>
+      <c r="J190" s="2" t="inlineStr">
+        <is>
+          <t>353724</t>
+        </is>
+      </c>
+      <c r="K190" s="2" t="inlineStr">
+        <is>
+          <t>1083077</t>
+        </is>
+      </c>
+      <c r="L190" s="2" t="inlineStr">
+        <is>
+          <t>772.4741148204537</t>
+        </is>
+      </c>
+      <c r="M190" s="2" t="inlineStr">
+        <is>
+          <t>105329.84546246429</t>
+        </is>
+      </c>
+      <c r="N190" s="2" t="inlineStr">
+        <is>
+          <t>350069.08271772147</t>
+        </is>
+      </c>
+      <c r="O190" s="2" t="inlineStr">
+        <is>
+          <t>901783.7910637569</t>
+        </is>
+      </c>
+      <c r="P190" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q190" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R190" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S190" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T190" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U190" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V190" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W190" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X190" s="2" t="inlineStr">
+        <is>
+          <t>6821143.069999966</t>
+        </is>
+      </c>
+      <c r="Y190" s="2" t="inlineStr">
+        <is>
+          <t>114262640.09325212</t>
+        </is>
+      </c>
+      <c r="Z190" s="2" t="inlineStr">
+        <is>
+          <t>479887356.656221</t>
+        </is>
+      </c>
+      <c r="AA190" s="2" t="inlineStr">
+        <is>
+          <t>1469620100.0734105</t>
+        </is>
+      </c>
+      <c r="AB190" s="2" t="inlineStr">
+        <is>
+          <t>7202</t>
+        </is>
+      </c>
+      <c r="AC190" s="2" t="inlineStr">
+        <is>
+          <t>62811</t>
+        </is>
+      </c>
+      <c r="AD190" s="2" t="inlineStr">
+        <is>
+          <t>273789</t>
+        </is>
+      </c>
+      <c r="AE190" s="2" t="inlineStr">
+        <is>
+          <t>765617</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-10-27
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE190"/>
+  <dimension ref="A1:AE191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30302,6 +30302,163 @@
         </is>
       </c>
     </row>
+    <row r="191">
+      <c r="A191" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B191" s="2" t="inlineStr">
+        <is>
+          <t>33583641119.707695</t>
+        </is>
+      </c>
+      <c r="C191" s="2" t="inlineStr">
+        <is>
+          <t>2320888061.9516697</t>
+        </is>
+      </c>
+      <c r="D191" s="2" t="inlineStr">
+        <is>
+          <t>81548</t>
+        </is>
+      </c>
+      <c r="E191" s="2" t="inlineStr">
+        <is>
+          <t>2319991860.270352</t>
+        </is>
+      </c>
+      <c r="F191" s="2" t="inlineStr">
+        <is>
+          <t>25726473754.820004</t>
+        </is>
+      </c>
+      <c r="G191" s="2" t="inlineStr">
+        <is>
+          <t>408264</t>
+        </is>
+      </c>
+      <c r="H191" s="2" t="inlineStr">
+        <is>
+          <t>12036</t>
+        </is>
+      </c>
+      <c r="I191" s="2" t="inlineStr">
+        <is>
+          <t>69670</t>
+        </is>
+      </c>
+      <c r="J191" s="2" t="inlineStr">
+        <is>
+          <t>358390</t>
+        </is>
+      </c>
+      <c r="K191" s="2" t="inlineStr">
+        <is>
+          <t>1078692</t>
+        </is>
+      </c>
+      <c r="L191" s="2" t="inlineStr">
+        <is>
+          <t>5282.094729887277</t>
+        </is>
+      </c>
+      <c r="M191" s="2" t="inlineStr">
+        <is>
+          <t>108353.13268527789</t>
+        </is>
+      </c>
+      <c r="N191" s="2" t="inlineStr">
+        <is>
+          <t>362365.04778607487</t>
+        </is>
+      </c>
+      <c r="O191" s="2" t="inlineStr">
+        <is>
+          <t>903870.585465251</t>
+        </is>
+      </c>
+      <c r="P191" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q191" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R191" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S191" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T191" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U191" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V191" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W191" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X191" s="2" t="inlineStr">
+        <is>
+          <t>1912656.6499999994</t>
+        </is>
+      </c>
+      <c r="Y191" s="2" t="inlineStr">
+        <is>
+          <t>122813215.60325213</t>
+        </is>
+      </c>
+      <c r="Z191" s="2" t="inlineStr">
+        <is>
+          <t>493232800.9377856</t>
+        </is>
+      </c>
+      <c r="AA191" s="2" t="inlineStr">
+        <is>
+          <t>1473349350.1534104</t>
+        </is>
+      </c>
+      <c r="AB191" s="2" t="inlineStr">
+        <is>
+          <t>257</t>
+        </is>
+      </c>
+      <c r="AC191" s="2" t="inlineStr">
+        <is>
+          <t>64740</t>
+        </is>
+      </c>
+      <c r="AD191" s="2" t="inlineStr">
+        <is>
+          <t>274495</t>
+        </is>
+      </c>
+      <c r="AE191" s="2" t="inlineStr">
+        <is>
+          <t>766304</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-10-28
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE191"/>
+  <dimension ref="A1:AE192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30459,6 +30459,163 @@
         </is>
       </c>
     </row>
+    <row r="192">
+      <c r="A192" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B192" s="2" t="inlineStr">
+        <is>
+          <t>33691097719.941013</t>
+        </is>
+      </c>
+      <c r="C192" s="2" t="inlineStr">
+        <is>
+          <t>2323206256.439465</t>
+        </is>
+      </c>
+      <c r="D192" s="2" t="inlineStr">
+        <is>
+          <t>81574</t>
+        </is>
+      </c>
+      <c r="E192" s="2" t="inlineStr">
+        <is>
+          <t>2323182743.245211</t>
+        </is>
+      </c>
+      <c r="F192" s="2" t="inlineStr">
+        <is>
+          <t>25817659078.919983</t>
+        </is>
+      </c>
+      <c r="G192" s="2" t="inlineStr">
+        <is>
+          <t>409133</t>
+        </is>
+      </c>
+      <c r="H192" s="2" t="inlineStr">
+        <is>
+          <t>9465</t>
+        </is>
+      </c>
+      <c r="I192" s="2" t="inlineStr">
+        <is>
+          <t>69136</t>
+        </is>
+      </c>
+      <c r="J192" s="2" t="inlineStr">
+        <is>
+          <t>366097</t>
+        </is>
+      </c>
+      <c r="K192" s="2" t="inlineStr">
+        <is>
+          <t>1080489</t>
+        </is>
+      </c>
+      <c r="L192" s="2" t="inlineStr">
+        <is>
+          <t>4496.256821135141</t>
+        </is>
+      </c>
+      <c r="M192" s="2" t="inlineStr">
+        <is>
+          <t>108200.88052001137</t>
+        </is>
+      </c>
+      <c r="N192" s="2" t="inlineStr">
+        <is>
+          <t>383840.1215876601</t>
+        </is>
+      </c>
+      <c r="O192" s="2" t="inlineStr">
+        <is>
+          <t>917615.9152666973</t>
+        </is>
+      </c>
+      <c r="P192" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q192" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R192" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S192" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T192" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U192" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V192" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W192" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X192" s="2" t="inlineStr">
+        <is>
+          <t>9373628.18</t>
+        </is>
+      </c>
+      <c r="Y192" s="2" t="inlineStr">
+        <is>
+          <t>119595443.71325213</t>
+        </is>
+      </c>
+      <c r="Z192" s="2" t="inlineStr">
+        <is>
+          <t>503585715.6677856</t>
+        </is>
+      </c>
+      <c r="AA192" s="2" t="inlineStr">
+        <is>
+          <t>1476328137.3834105</t>
+        </is>
+      </c>
+      <c r="AB192" s="2" t="inlineStr">
+        <is>
+          <t>9274</t>
+        </is>
+      </c>
+      <c r="AC192" s="2" t="inlineStr">
+        <is>
+          <t>64418</t>
+        </is>
+      </c>
+      <c r="AD192" s="2" t="inlineStr">
+        <is>
+          <t>275246</t>
+        </is>
+      </c>
+      <c r="AE192" s="2" t="inlineStr">
+        <is>
+          <t>768414</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-10-29
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE192"/>
+  <dimension ref="A1:AE193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30616,6 +30616,163 @@
         </is>
       </c>
     </row>
+    <row r="193">
+      <c r="A193" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B193" s="2" t="inlineStr">
+        <is>
+          <t>33787681020.444923</t>
+        </is>
+      </c>
+      <c r="C193" s="2" t="inlineStr">
+        <is>
+          <t>2330704001.658251</t>
+        </is>
+      </c>
+      <c r="D193" s="2" t="inlineStr">
+        <is>
+          <t>81605</t>
+        </is>
+      </c>
+      <c r="E193" s="2" t="inlineStr">
+        <is>
+          <t>2325315751.407324</t>
+        </is>
+      </c>
+      <c r="F193" s="2" t="inlineStr">
+        <is>
+          <t>25889617121.13001</t>
+        </is>
+      </c>
+      <c r="G193" s="2" t="inlineStr">
+        <is>
+          <t>409922</t>
+        </is>
+      </c>
+      <c r="H193" s="2" t="inlineStr">
+        <is>
+          <t>9275</t>
+        </is>
+      </c>
+      <c r="I193" s="2" t="inlineStr">
+        <is>
+          <t>69952</t>
+        </is>
+      </c>
+      <c r="J193" s="2" t="inlineStr">
+        <is>
+          <t>363406</t>
+        </is>
+      </c>
+      <c r="K193" s="2" t="inlineStr">
+        <is>
+          <t>1081816</t>
+        </is>
+      </c>
+      <c r="L193" s="2" t="inlineStr">
+        <is>
+          <t>4008.9914887575646</t>
+        </is>
+      </c>
+      <c r="M193" s="2" t="inlineStr">
+        <is>
+          <t>111209.3743417058</t>
+        </is>
+      </c>
+      <c r="N193" s="2" t="inlineStr">
+        <is>
+          <t>396997.09387838084</t>
+        </is>
+      </c>
+      <c r="O193" s="2" t="inlineStr">
+        <is>
+          <t>926855.6368906343</t>
+        </is>
+      </c>
+      <c r="P193" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q193" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R193" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S193" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T193" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U193" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V193" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W193" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X193" s="2" t="inlineStr">
+        <is>
+          <t>6999361.492915497</t>
+        </is>
+      </c>
+      <c r="Y193" s="2" t="inlineStr">
+        <is>
+          <t>126948559.76831755</t>
+        </is>
+      </c>
+      <c r="Z193" s="2" t="inlineStr">
+        <is>
+          <t>512875372.00778556</t>
+        </is>
+      </c>
+      <c r="AA193" s="2" t="inlineStr">
+        <is>
+          <t>1482000740.2784104</t>
+        </is>
+      </c>
+      <c r="AB193" s="2" t="inlineStr">
+        <is>
+          <t>7167</t>
+        </is>
+      </c>
+      <c r="AC193" s="2" t="inlineStr">
+        <is>
+          <t>65843</t>
+        </is>
+      </c>
+      <c r="AD193" s="2" t="inlineStr">
+        <is>
+          <t>276670</t>
+        </is>
+      </c>
+      <c r="AE193" s="2" t="inlineStr">
+        <is>
+          <t>771332</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-10-30
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE193"/>
+  <dimension ref="A1:AE194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30773,6 +30773,163 @@
         </is>
       </c>
     </row>
+    <row r="194">
+      <c r="A194" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B194" s="2" t="inlineStr">
+        <is>
+          <t>33863172727.658234</t>
+        </is>
+      </c>
+      <c r="C194" s="2" t="inlineStr">
+        <is>
+          <t>2335566299.8046064</t>
+        </is>
+      </c>
+      <c r="D194" s="2" t="inlineStr">
+        <is>
+          <t>81623</t>
+        </is>
+      </c>
+      <c r="E194" s="2" t="inlineStr">
+        <is>
+          <t>2334987805.4866047</t>
+        </is>
+      </c>
+      <c r="F194" s="2" t="inlineStr">
+        <is>
+          <t>25936042606.519997</t>
+        </is>
+      </c>
+      <c r="G194" s="2" t="inlineStr">
+        <is>
+          <t>410414</t>
+        </is>
+      </c>
+      <c r="H194" s="2" t="inlineStr">
+        <is>
+          <t>8480</t>
+        </is>
+      </c>
+      <c r="I194" s="2" t="inlineStr">
+        <is>
+          <t>72550</t>
+        </is>
+      </c>
+      <c r="J194" s="2" t="inlineStr">
+        <is>
+          <t>364979</t>
+        </is>
+      </c>
+      <c r="K194" s="2" t="inlineStr">
+        <is>
+          <t>1089241</t>
+        </is>
+      </c>
+      <c r="L194" s="2" t="inlineStr">
+        <is>
+          <t>3962.7669554476356</t>
+        </is>
+      </c>
+      <c r="M194" s="2" t="inlineStr">
+        <is>
+          <t>110488.44687003836</t>
+        </is>
+      </c>
+      <c r="N194" s="2" t="inlineStr">
+        <is>
+          <t>403279.3036004399</t>
+        </is>
+      </c>
+      <c r="O194" s="2" t="inlineStr">
+        <is>
+          <t>935260.7202794233</t>
+        </is>
+      </c>
+      <c r="P194" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q194" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R194" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S194" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T194" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U194" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V194" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W194" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X194" s="2" t="inlineStr">
+        <is>
+          <t>9471284.150000012</t>
+        </is>
+      </c>
+      <c r="Y194" s="2" t="inlineStr">
+        <is>
+          <t>132659828.85861595</t>
+        </is>
+      </c>
+      <c r="Z194" s="2" t="inlineStr">
+        <is>
+          <t>522506572.2207011</t>
+        </is>
+      </c>
+      <c r="AA194" s="2" t="inlineStr">
+        <is>
+          <t>1494046611.541326</t>
+        </is>
+      </c>
+      <c r="AB194" s="2" t="inlineStr">
+        <is>
+          <t>8931</t>
+        </is>
+      </c>
+      <c r="AC194" s="2" t="inlineStr">
+        <is>
+          <t>64928</t>
+        </is>
+      </c>
+      <c r="AD194" s="2" t="inlineStr">
+        <is>
+          <t>277722</t>
+        </is>
+      </c>
+      <c r="AE194" s="2" t="inlineStr">
+        <is>
+          <t>776812</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily pulse data: 2026-10-31
</commit_message>
<xml_diff>
--- a/provenance_pulse_tracker.xlsx
+++ b/provenance_pulse_tracker.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE194"/>
+  <dimension ref="A1:AE195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30930,6 +30930,163 @@
         </is>
       </c>
     </row>
+    <row r="195">
+      <c r="A195" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B195" s="2" t="inlineStr">
+        <is>
+          <t>33947255061.020687</t>
+        </is>
+      </c>
+      <c r="C195" s="2" t="inlineStr">
+        <is>
+          <t>2320374442.3364887</t>
+        </is>
+      </c>
+      <c r="D195" s="2" t="inlineStr">
+        <is>
+          <t>81653</t>
+        </is>
+      </c>
+      <c r="E195" s="2" t="inlineStr">
+        <is>
+          <t>2320058514.4541826</t>
+        </is>
+      </c>
+      <c r="F195" s="2" t="inlineStr">
+        <is>
+          <t>26019537761.189995</t>
+        </is>
+      </c>
+      <c r="G195" s="2" t="inlineStr">
+        <is>
+          <t>411407</t>
+        </is>
+      </c>
+      <c r="H195" s="2" t="inlineStr">
+        <is>
+          <t>8864</t>
+        </is>
+      </c>
+      <c r="I195" s="2" t="inlineStr">
+        <is>
+          <t>77243</t>
+        </is>
+      </c>
+      <c r="J195" s="2" t="inlineStr">
+        <is>
+          <t>365672</t>
+        </is>
+      </c>
+      <c r="K195" s="2" t="inlineStr">
+        <is>
+          <t>1098500</t>
+        </is>
+      </c>
+      <c r="L195" s="2" t="inlineStr">
+        <is>
+          <t>3764.143096992489</t>
+        </is>
+      </c>
+      <c r="M195" s="2" t="inlineStr">
+        <is>
+          <t>114578.57972334149</t>
+        </is>
+      </c>
+      <c r="N195" s="2" t="inlineStr">
+        <is>
+          <t>415299.6573738526</t>
+        </is>
+      </c>
+      <c r="O195" s="2" t="inlineStr">
+        <is>
+          <t>952982.4370529151</t>
+        </is>
+      </c>
+      <c r="P195" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="Q195" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="R195" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="S195" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="T195" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="U195" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="V195" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="W195" s="2" t="inlineStr">
+        <is>
+          <t>HTTP 400</t>
+        </is>
+      </c>
+      <c r="X195" s="2" t="inlineStr">
+        <is>
+          <t>2267033.389999999</t>
+        </is>
+      </c>
+      <c r="Y195" s="2" t="inlineStr">
+        <is>
+          <t>139388058.298616</t>
+        </is>
+      </c>
+      <c r="Z195" s="2" t="inlineStr">
+        <is>
+          <t>526461363.3271961</t>
+        </is>
+      </c>
+      <c r="AA195" s="2" t="inlineStr">
+        <is>
+          <t>1506094416.021326</t>
+        </is>
+      </c>
+      <c r="AB195" s="2" t="inlineStr">
+        <is>
+          <t>1638</t>
+        </is>
+      </c>
+      <c r="AC195" s="2" t="inlineStr">
+        <is>
+          <t>66009</t>
+        </is>
+      </c>
+      <c r="AD195" s="2" t="inlineStr">
+        <is>
+          <t>279104</t>
+        </is>
+      </c>
+      <c r="AE195" s="2" t="inlineStr">
+        <is>
+          <t>778094</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>